<commit_message>
29 Sep 1er Parcial
</commit_message>
<xml_diff>
--- a/Totales Generales.xlsx
+++ b/Totales Generales.xlsx
@@ -68,103 +68,103 @@
     <t>Grupo</t>
   </si>
   <si>
-    <t>2AEM</t>
-  </si>
-  <si>
-    <t>2ALCM</t>
-  </si>
-  <si>
-    <t>2APM</t>
-  </si>
-  <si>
-    <t>2ARHM</t>
-  </si>
-  <si>
-    <t>2BEM</t>
-  </si>
-  <si>
-    <t>2BLCM</t>
-  </si>
-  <si>
-    <t>4AEM</t>
-  </si>
-  <si>
-    <t>4ALCM</t>
-  </si>
-  <si>
-    <t>4APM</t>
-  </si>
-  <si>
-    <t>4ARHM</t>
-  </si>
-  <si>
-    <t>4BEM</t>
-  </si>
-  <si>
-    <t>4BLCM</t>
-  </si>
-  <si>
-    <t>6AEM</t>
-  </si>
-  <si>
-    <t>6ALCM</t>
-  </si>
-  <si>
-    <t>6APM</t>
-  </si>
-  <si>
-    <t>6ARHM</t>
-  </si>
-  <si>
-    <t>6BEM</t>
-  </si>
-  <si>
-    <t>6BLCM</t>
-  </si>
-  <si>
-    <t>2AEV</t>
-  </si>
-  <si>
-    <t>2ALCV</t>
-  </si>
-  <si>
-    <t>2APV</t>
-  </si>
-  <si>
-    <t>2ARHV</t>
-  </si>
-  <si>
-    <t>2ASV</t>
-  </si>
-  <si>
-    <t>4AEV</t>
-  </si>
-  <si>
-    <t>4ALCV</t>
-  </si>
-  <si>
-    <t>4APV</t>
-  </si>
-  <si>
-    <t>4ARHV</t>
-  </si>
-  <si>
-    <t>4ASV</t>
-  </si>
-  <si>
-    <t>6AEV</t>
-  </si>
-  <si>
-    <t>6ALCV</t>
-  </si>
-  <si>
-    <t>6APV</t>
-  </si>
-  <si>
-    <t>6ARHV</t>
-  </si>
-  <si>
-    <t>6ASV</t>
+    <t>1AM</t>
+  </si>
+  <si>
+    <t>1BM</t>
+  </si>
+  <si>
+    <t>1CM</t>
+  </si>
+  <si>
+    <t>1DM</t>
+  </si>
+  <si>
+    <t>1EM</t>
+  </si>
+  <si>
+    <t>1FM</t>
+  </si>
+  <si>
+    <t>3AEM</t>
+  </si>
+  <si>
+    <t>3ALCM</t>
+  </si>
+  <si>
+    <t>3APM</t>
+  </si>
+  <si>
+    <t>3ARHM</t>
+  </si>
+  <si>
+    <t>3BEM</t>
+  </si>
+  <si>
+    <t>3BLCM</t>
+  </si>
+  <si>
+    <t>5AEM</t>
+  </si>
+  <si>
+    <t>5ALCM</t>
+  </si>
+  <si>
+    <t>5APM</t>
+  </si>
+  <si>
+    <t>5ARHM</t>
+  </si>
+  <si>
+    <t>5BEM</t>
+  </si>
+  <si>
+    <t>5BLCM</t>
+  </si>
+  <si>
+    <t>1AV</t>
+  </si>
+  <si>
+    <t>1BV</t>
+  </si>
+  <si>
+    <t>1CV</t>
+  </si>
+  <si>
+    <t>1DV</t>
+  </si>
+  <si>
+    <t>1EV</t>
+  </si>
+  <si>
+    <t>3AEV</t>
+  </si>
+  <si>
+    <t>3ALCV</t>
+  </si>
+  <si>
+    <t>3APV</t>
+  </si>
+  <si>
+    <t>3ARHV</t>
+  </si>
+  <si>
+    <t>3ASV</t>
+  </si>
+  <si>
+    <t>5AEV</t>
+  </si>
+  <si>
+    <t>5ALCV</t>
+  </si>
+  <si>
+    <t>5APV</t>
+  </si>
+  <si>
+    <t>5ARHV</t>
+  </si>
+  <si>
+    <t>5ASV</t>
   </si>
   <si>
     <t>Apro1P</t>
@@ -586,248 +586,248 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
       </c>
       <c r="C2">
-        <v>216</v>
+        <v>234</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G2">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I2">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="J2">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="K2">
-        <v>152</v>
+        <v>129</v>
       </c>
       <c r="L2">
-        <v>64</v>
+        <v>105</v>
       </c>
       <c r="M2">
-        <v>29.63</v>
+        <v>44.87</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>8</v>
       </c>
       <c r="H3">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I3">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="J3">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="K3">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="L3">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="M3">
-        <v>39.69</v>
+        <v>35.19</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
       <c r="C4">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I4">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="J4">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="K4">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="L4">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="M4">
-        <v>32.97</v>
+        <v>44.62</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
       <c r="C5">
-        <v>164</v>
+        <v>191</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G5">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="H5">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="J5">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="K5">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="L5">
-        <v>75</v>
+        <v>107</v>
       </c>
       <c r="M5">
-        <v>45.73</v>
+        <v>56.02</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G6">
         <v>10</v>
       </c>
       <c r="H6">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I6">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J6">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="K6">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="L6">
-        <v>70</v>
+        <v>136</v>
       </c>
       <c r="M6">
-        <v>51.85</v>
+        <v>88.89</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7">
-        <v>148</v>
+        <v>130</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G7">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H7">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="I7">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="J7">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K7">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="L7">
-        <v>63</v>
+        <v>115</v>
       </c>
       <c r="M7">
-        <v>42.57</v>
+        <v>88.45999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -883,248 +883,248 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
       </c>
       <c r="C2">
-        <v>216</v>
+        <v>234</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>234</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>162</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>54</v>
+        <v>234</v>
       </c>
       <c r="M2">
-        <v>25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>215</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>82</v>
+        <v>216</v>
       </c>
       <c r="M3">
-        <v>42.27</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
       <c r="C4">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>125</v>
       </c>
       <c r="F4">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>115</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>67</v>
+        <v>186</v>
       </c>
       <c r="M4">
-        <v>36.81</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
       <c r="C5">
-        <v>164</v>
+        <v>191</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>191</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="K5">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>73</v>
+        <v>191</v>
       </c>
       <c r="M5">
-        <v>44.51</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>144</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
         <v>6</v>
       </c>
-      <c r="I6">
-        <v>13</v>
-      </c>
       <c r="J6">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="K6">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <v>65</v>
+        <v>153</v>
       </c>
       <c r="M6">
-        <v>48.15</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7">
-        <v>148</v>
+        <v>130</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>95</v>
       </c>
       <c r="F7">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G7">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I7">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="J7">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="M7">
-        <v>48.65</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1180,248 +1180,248 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
       </c>
       <c r="C2">
-        <v>216</v>
+        <v>234</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="K2">
-        <v>202</v>
+        <v>129</v>
       </c>
       <c r="L2">
-        <v>14</v>
+        <v>105</v>
       </c>
       <c r="M2">
-        <v>6.48</v>
+        <v>44.87</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="J3">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="K3">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="L3">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="M3">
-        <v>19.59</v>
+        <v>35.19</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
       <c r="C4">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="I4">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="J4">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="K4">
-        <v>171</v>
+        <v>103</v>
       </c>
       <c r="L4">
-        <v>11</v>
+        <v>83</v>
       </c>
       <c r="M4">
-        <v>6.04</v>
+        <v>44.62</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
       <c r="C5">
-        <v>164</v>
+        <v>191</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="H5">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="I5">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="J5">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="K5">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="L5">
-        <v>45</v>
+        <v>107</v>
       </c>
       <c r="M5">
-        <v>27.44</v>
+        <v>56.02</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="I6">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="J6">
+        <v>80</v>
+      </c>
+      <c r="K6">
         <v>17</v>
       </c>
-      <c r="K6">
-        <v>95</v>
-      </c>
       <c r="L6">
-        <v>40</v>
+        <v>136</v>
       </c>
       <c r="M6">
-        <v>29.63</v>
+        <v>88.89</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7">
-        <v>148</v>
+        <v>130</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="I7">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="J7">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="K7">
-        <v>118</v>
+        <v>15</v>
       </c>
       <c r="L7">
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="M7">
-        <v>20.27</v>
+        <v>88.45999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1477,7 +1477,7 @@
         <v>16</v>
       </c>
       <c r="B2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1486,28 +1486,28 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J2">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>47.06</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -1515,37 +1515,37 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="K3">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="L3">
-        <v>11.36</v>
+        <v>48.39</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1553,7 +1553,7 @@
         <v>18</v>
       </c>
       <c r="B4">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1568,22 +1568,22 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J4">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="L4">
-        <v>3.7</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1591,7 +1591,7 @@
         <v>19</v>
       </c>
       <c r="B5">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -1603,25 +1603,25 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5">
         <v>2</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J5">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K5">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L5">
-        <v>13.51</v>
+        <v>20.45</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -1629,7 +1629,7 @@
         <v>20</v>
       </c>
       <c r="B6">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1638,28 +1638,28 @@
         <v>0</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J6">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="K6">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="L6">
-        <v>6.25</v>
+        <v>72.09</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -1667,37 +1667,37 @@
         <v>21</v>
       </c>
       <c r="B7">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J7">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="L7">
-        <v>2.27</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -1717,25 +1717,25 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I8">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J8">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="K8">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L8">
-        <v>28.13</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -1743,7 +1743,7 @@
         <v>23</v>
       </c>
       <c r="B9">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -1752,28 +1752,28 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9">
         <v>0</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J9">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="K9">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="L9">
-        <v>8.33</v>
+        <v>31.71</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1781,37 +1781,37 @@
         <v>24</v>
       </c>
       <c r="B10">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>2</v>
+      </c>
+      <c r="J10">
         <v>24</v>
       </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>2</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10">
-        <v>22</v>
-      </c>
       <c r="K10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10">
-        <v>8.33</v>
+        <v>11.11</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1819,37 +1819,37 @@
         <v>25</v>
       </c>
       <c r="B11">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C11">
         <v>0</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11">
         <v>2</v>
       </c>
       <c r="H11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11">
         <v>4</v>
       </c>
       <c r="J11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="K11">
         <v>10</v>
       </c>
       <c r="L11">
-        <v>27.78</v>
+        <v>25.64</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1857,37 +1857,37 @@
         <v>26</v>
       </c>
       <c r="B12">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
         <v>3</v>
       </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
       <c r="G12">
         <v>2</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I12">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J12">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="K12">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="L12">
-        <v>30.3</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1895,37 +1895,37 @@
         <v>27</v>
       </c>
       <c r="B13">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G13">
         <v>0</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I13">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="J13">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K13">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="L13">
-        <v>12.12</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1933,7 +1933,7 @@
         <v>28</v>
       </c>
       <c r="B14">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1945,25 +1945,25 @@
         <v>1</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="J14">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="K14">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="L14">
-        <v>21.05</v>
+        <v>70.97</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1971,7 +1971,7 @@
         <v>29</v>
       </c>
       <c r="B15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1986,22 +1986,22 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J15">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="K15">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L15">
-        <v>2.94</v>
+        <v>25.71</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -2009,7 +2009,7 @@
         <v>30</v>
       </c>
       <c r="B16">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -2021,25 +2021,25 @@
         <v>0</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J16">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="K16">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L16">
-        <v>4.17</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -2047,7 +2047,7 @@
         <v>31</v>
       </c>
       <c r="B17">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -2059,25 +2059,25 @@
         <v>0</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J17">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="K17">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L17">
-        <v>0</v>
+        <v>32.43</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -2085,37 +2085,37 @@
         <v>32</v>
       </c>
       <c r="B18">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18">
         <v>0</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J18">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="K18">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="L18">
-        <v>3.23</v>
+        <v>53.33</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -2123,7 +2123,7 @@
         <v>33</v>
       </c>
       <c r="B19">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -2138,22 +2138,22 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J19">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="K19">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L19">
-        <v>0</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -2161,37 +2161,37 @@
         <v>34</v>
       </c>
       <c r="B20">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I20">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J20">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="K20">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="L20">
-        <v>36.11</v>
+        <v>61.54</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -2199,37 +2199,37 @@
         <v>35</v>
       </c>
       <c r="B21">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E21">
         <v>0</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I21">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J21">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="K21">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="L21">
-        <v>22.5</v>
+        <v>58.82</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -2237,37 +2237,37 @@
         <v>36</v>
       </c>
       <c r="B22">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C22">
         <v>0</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J22">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="K22">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="L22">
-        <v>28.57</v>
+        <v>39.02</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -2281,31 +2281,31 @@
         <v>0</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I23">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="J23">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="K23">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="L23">
-        <v>34.15</v>
+        <v>63.41</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -2313,7 +2313,7 @@
         <v>38</v>
       </c>
       <c r="B24">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -2325,25 +2325,25 @@
         <v>0</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I24">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="J24">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="K24">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="L24">
-        <v>5.26</v>
+        <v>58.33</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -2351,37 +2351,37 @@
         <v>39</v>
       </c>
       <c r="B25">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I25">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="J25">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="K25">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="L25">
-        <v>41.94</v>
+        <v>87.18000000000001</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -2389,37 +2389,37 @@
         <v>40</v>
       </c>
       <c r="B26">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C26">
         <v>0</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26">
         <v>1</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I26">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="J26">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="K26">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="L26">
-        <v>26.67</v>
+        <v>97.44</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -2427,37 +2427,37 @@
         <v>41</v>
       </c>
       <c r="B27">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27">
         <v>3</v>
       </c>
-      <c r="D27">
-        <v>1</v>
-      </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
       <c r="F27">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H27">
         <v>1</v>
       </c>
       <c r="I27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J27">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K27">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="L27">
-        <v>50</v>
+        <v>60.71</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -2465,37 +2465,37 @@
         <v>42</v>
       </c>
       <c r="B28">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C28">
         <v>0</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E28">
         <v>0</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H28">
         <v>1</v>
       </c>
       <c r="I28">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
         <v>32</v>
       </c>
-      <c r="K28">
-        <v>3</v>
-      </c>
       <c r="L28">
-        <v>8.57</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -2503,37 +2503,37 @@
         <v>43</v>
       </c>
       <c r="B29">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C29">
         <v>0</v>
       </c>
       <c r="D29">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I29">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J29">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K29">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="L29">
-        <v>31.58</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -2541,37 +2541,37 @@
         <v>44</v>
       </c>
       <c r="B30">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C30">
         <v>0</v>
       </c>
       <c r="D30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H30">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J30">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="K30">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="L30">
-        <v>26.32</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -2579,7 +2579,7 @@
         <v>45</v>
       </c>
       <c r="B31">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -2588,28 +2588,28 @@
         <v>0</v>
       </c>
       <c r="E31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31">
         <v>0</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H31">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I31">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J31">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="K31">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="L31">
-        <v>6.25</v>
+        <v>77.78</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -2617,37 +2617,37 @@
         <v>46</v>
       </c>
       <c r="B32">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C32">
         <v>0</v>
       </c>
       <c r="D32">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32">
         <v>0</v>
       </c>
       <c r="G32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H32">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I32">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J32">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="K32">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L32">
-        <v>28.13</v>
+        <v>57.89</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -2655,37 +2655,37 @@
         <v>47</v>
       </c>
       <c r="B33">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C33">
         <v>0</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G33">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I33">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J33">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="K33">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="L33">
-        <v>18.18</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -2693,7 +2693,7 @@
         <v>48</v>
       </c>
       <c r="B34">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -2702,28 +2702,28 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G34">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H34">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I34">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J34">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K34">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="L34">
-        <v>25</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2767,25 +2767,25 @@
         <v>16</v>
       </c>
       <c r="B2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C2">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D2">
-        <v>81.25</v>
+        <v>52.94</v>
       </c>
       <c r="E2">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>78.13</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="H2">
-        <v>100</v>
+        <v>52.94</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2793,25 +2793,25 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C3">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D3">
-        <v>65.91</v>
+        <v>51.61</v>
       </c>
       <c r="E3">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>72.73</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="H3">
-        <v>88.64</v>
+        <v>51.61</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2819,25 +2819,25 @@
         <v>18</v>
       </c>
       <c r="B4">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="C4">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4">
-        <v>81.48</v>
+        <v>60</v>
       </c>
       <c r="E4">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>77.78</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H4">
-        <v>96.3</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2845,25 +2845,25 @@
         <v>19</v>
       </c>
       <c r="B5">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C5">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D5">
-        <v>89.19</v>
+        <v>79.55</v>
       </c>
       <c r="E5">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>81.08</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H5">
-        <v>86.48999999999999</v>
+        <v>79.55</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2871,25 +2871,25 @@
         <v>20</v>
       </c>
       <c r="B6">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="C6">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D6">
-        <v>53.13</v>
+        <v>27.91</v>
       </c>
       <c r="E6">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>65.63</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="H6">
-        <v>93.75</v>
+        <v>27.91</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -2897,25 +2897,25 @@
         <v>21</v>
       </c>
       <c r="B7">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C7">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D7">
-        <v>56.82</v>
+        <v>57.14</v>
       </c>
       <c r="E7">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="H7">
-        <v>97.73</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2926,22 +2926,22 @@
         <v>32</v>
       </c>
       <c r="C8">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D8">
-        <v>46.88</v>
+        <v>62.5</v>
       </c>
       <c r="E8">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F8">
-        <v>59.38</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H8">
-        <v>71.88</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2949,25 +2949,25 @@
         <v>23</v>
       </c>
       <c r="B9">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C9">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D9">
-        <v>75</v>
+        <v>68.29000000000001</v>
       </c>
       <c r="E9">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>69.44</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H9">
-        <v>91.67</v>
+        <v>68.29000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2975,25 +2975,25 @@
         <v>24</v>
       </c>
       <c r="B10">
+        <v>27</v>
+      </c>
+      <c r="C10">
         <v>24</v>
       </c>
-      <c r="C10">
-        <v>13</v>
-      </c>
       <c r="D10">
-        <v>54.17</v>
+        <v>88.89</v>
       </c>
       <c r="E10">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F10">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H10">
-        <v>91.67</v>
+        <v>88.89</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -3001,25 +3001,25 @@
         <v>25</v>
       </c>
       <c r="B11">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C11">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D11">
-        <v>69.44</v>
+        <v>74.36</v>
       </c>
       <c r="E11">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>52.78</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="H11">
-        <v>72.22</v>
+        <v>74.36</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -3027,25 +3027,25 @@
         <v>26</v>
       </c>
       <c r="B12">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C12">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D12">
-        <v>42.42</v>
+        <v>37.5</v>
       </c>
       <c r="E12">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>51.52</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="H12">
-        <v>69.7</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -3053,25 +3053,25 @@
         <v>27</v>
       </c>
       <c r="B13">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="C13">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D13">
-        <v>69.7</v>
+        <v>60</v>
       </c>
       <c r="E13">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>60.61</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H13">
-        <v>87.88</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -3079,25 +3079,25 @@
         <v>28</v>
       </c>
       <c r="B14">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C14">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="D14">
-        <v>60.53</v>
+        <v>29.03</v>
       </c>
       <c r="E14">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>42.11</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="H14">
-        <v>78.95</v>
+        <v>29.03</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -3105,25 +3105,25 @@
         <v>29</v>
       </c>
       <c r="B15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C15">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D15">
-        <v>70.59</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="E15">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="F15">
-        <v>91.18000000000001</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="H15">
-        <v>97.06</v>
+        <v>74.29000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -3131,25 +3131,25 @@
         <v>30</v>
       </c>
       <c r="B16">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C16">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D16">
-        <v>50</v>
+        <v>42.86</v>
       </c>
       <c r="E16">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>33.33</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="H16">
-        <v>95.83</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -3157,25 +3157,25 @@
         <v>31</v>
       </c>
       <c r="B17">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="C17">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D17">
-        <v>77.27</v>
+        <v>67.56999999999999</v>
       </c>
       <c r="E17">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F17">
-        <v>72.73</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H17">
-        <v>100</v>
+        <v>67.56999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -3183,25 +3183,25 @@
         <v>32</v>
       </c>
       <c r="B18">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D18">
-        <v>54.84</v>
+        <v>46.67</v>
       </c>
       <c r="E18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F18">
-        <v>41.94</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="H18">
-        <v>96.77</v>
+        <v>46.67</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -3209,25 +3209,25 @@
         <v>33</v>
       </c>
       <c r="B19">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C19">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D19">
-        <v>87.88</v>
+        <v>62.5</v>
       </c>
       <c r="E19">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="F19">
-        <v>93.94</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="H19">
-        <v>100</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -3235,25 +3235,25 @@
         <v>34</v>
       </c>
       <c r="B20">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C20">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D20">
-        <v>38.89</v>
+        <v>38.46</v>
       </c>
       <c r="E20">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F20">
-        <v>44.44</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="H20">
-        <v>63.89</v>
+        <v>38.46</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -3261,25 +3261,25 @@
         <v>35</v>
       </c>
       <c r="B21">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C21">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D21">
-        <v>55</v>
+        <v>41.18</v>
       </c>
       <c r="E21">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F21">
-        <v>62.5</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="H21">
-        <v>77.5</v>
+        <v>41.18</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -3287,25 +3287,25 @@
         <v>36</v>
       </c>
       <c r="B22">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C22">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D22">
-        <v>60.71</v>
+        <v>60.98</v>
       </c>
       <c r="E22">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F22">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H22">
-        <v>71.43000000000001</v>
+        <v>60.98</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -3316,22 +3316,22 @@
         <v>41</v>
       </c>
       <c r="C23">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D23">
-        <v>58.54</v>
+        <v>36.59</v>
       </c>
       <c r="E23">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F23">
-        <v>58.54</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="H23">
-        <v>65.84999999999999</v>
+        <v>36.59</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -3339,25 +3339,25 @@
         <v>38</v>
       </c>
       <c r="B24">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="C24">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D24">
-        <v>63.16</v>
+        <v>41.67</v>
       </c>
       <c r="E24">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F24">
-        <v>63.16</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H24">
-        <v>94.73999999999999</v>
+        <v>41.67</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -3365,25 +3365,25 @@
         <v>39</v>
       </c>
       <c r="B25">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C25">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D25">
-        <v>25.81</v>
+        <v>12.82</v>
       </c>
       <c r="E25">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F25">
-        <v>29.03</v>
+        <v>0</v>
       </c>
       <c r="G25">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="H25">
-        <v>58.06</v>
+        <v>12.82</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -3391,25 +3391,25 @@
         <v>40</v>
       </c>
       <c r="B26">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C26">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="D26">
-        <v>73.33</v>
+        <v>2.56</v>
       </c>
       <c r="E26">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F26">
-        <v>73.33</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="H26">
-        <v>73.33</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -3417,25 +3417,25 @@
         <v>41</v>
       </c>
       <c r="B27">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C27">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D27">
-        <v>35</v>
+        <v>39.29</v>
       </c>
       <c r="E27">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F27">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H27">
-        <v>50</v>
+        <v>39.29</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -3443,25 +3443,25 @@
         <v>42</v>
       </c>
       <c r="B28">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C28">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>54.29</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F28">
-        <v>65.70999999999999</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="H28">
-        <v>91.43000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -3469,25 +3469,25 @@
         <v>43</v>
       </c>
       <c r="B29">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C29">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D29">
-        <v>47.37</v>
+        <v>0</v>
       </c>
       <c r="E29">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F29">
-        <v>52.63</v>
+        <v>0</v>
       </c>
       <c r="G29">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H29">
-        <v>68.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -3495,25 +3495,25 @@
         <v>44</v>
       </c>
       <c r="B30">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C30">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D30">
-        <v>31.58</v>
+        <v>0</v>
       </c>
       <c r="E30">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F30">
-        <v>36.84</v>
+        <v>0</v>
       </c>
       <c r="G30">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="H30">
-        <v>73.68000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -3521,25 +3521,25 @@
         <v>45</v>
       </c>
       <c r="B31">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C31">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="D31">
-        <v>71.88</v>
+        <v>22.22</v>
       </c>
       <c r="E31">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F31">
-        <v>71.88</v>
+        <v>0</v>
       </c>
       <c r="G31">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="H31">
-        <v>93.75</v>
+        <v>22.22</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -3547,25 +3547,25 @@
         <v>46</v>
       </c>
       <c r="B32">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C32">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="D32">
-        <v>53.13</v>
+        <v>42.11</v>
       </c>
       <c r="E32">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F32">
-        <v>40.63</v>
+        <v>0</v>
       </c>
       <c r="G32">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="H32">
-        <v>71.88</v>
+        <v>42.11</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -3573,25 +3573,25 @@
         <v>47</v>
       </c>
       <c r="B33">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C33">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D33">
-        <v>51.52</v>
+        <v>2.5</v>
       </c>
       <c r="E33">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F33">
-        <v>63.64</v>
+        <v>0</v>
       </c>
       <c r="G33">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="H33">
-        <v>81.81999999999999</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -3599,25 +3599,25 @@
         <v>48</v>
       </c>
       <c r="B34">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="C34">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D34">
-        <v>68.75</v>
+        <v>0</v>
       </c>
       <c r="E34">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F34">
-        <v>37.5</v>
+        <v>0</v>
       </c>
       <c r="G34">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="H34">
-        <v>75</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Primer Parcial con Asistencias
</commit_message>
<xml_diff>
--- a/Totales Generales.xlsx
+++ b/Totales Generales.xlsx
@@ -68,103 +68,103 @@
     <t>Grupo</t>
   </si>
   <si>
-    <t>1AM</t>
-  </si>
-  <si>
-    <t>1BM</t>
-  </si>
-  <si>
-    <t>1CM</t>
-  </si>
-  <si>
-    <t>1DM</t>
-  </si>
-  <si>
-    <t>1EM</t>
-  </si>
-  <si>
-    <t>1FM</t>
-  </si>
-  <si>
-    <t>3AEM</t>
-  </si>
-  <si>
-    <t>3ALCM</t>
-  </si>
-  <si>
-    <t>3APM</t>
-  </si>
-  <si>
-    <t>3ARHM</t>
-  </si>
-  <si>
-    <t>3BEM</t>
-  </si>
-  <si>
-    <t>3BLCM</t>
-  </si>
-  <si>
-    <t>5AEM</t>
-  </si>
-  <si>
-    <t>5ALCM</t>
-  </si>
-  <si>
-    <t>5APM</t>
-  </si>
-  <si>
-    <t>5ARHM</t>
-  </si>
-  <si>
-    <t>5BEM</t>
-  </si>
-  <si>
-    <t>5BLCM</t>
-  </si>
-  <si>
-    <t>1AV</t>
-  </si>
-  <si>
-    <t>1BV</t>
-  </si>
-  <si>
-    <t>1CV</t>
-  </si>
-  <si>
-    <t>1DV</t>
-  </si>
-  <si>
-    <t>1EV</t>
-  </si>
-  <si>
-    <t>3AEV</t>
-  </si>
-  <si>
-    <t>3ALCV</t>
-  </si>
-  <si>
-    <t>3APV</t>
-  </si>
-  <si>
-    <t>3ARHV</t>
-  </si>
-  <si>
-    <t>3ASV</t>
-  </si>
-  <si>
-    <t>5AEV</t>
-  </si>
-  <si>
-    <t>5ALCV</t>
-  </si>
-  <si>
-    <t>5APV</t>
-  </si>
-  <si>
-    <t>5ARHV</t>
-  </si>
-  <si>
-    <t>5ASV</t>
+    <t>2AEM</t>
+  </si>
+  <si>
+    <t>2ALCM</t>
+  </si>
+  <si>
+    <t>2APM</t>
+  </si>
+  <si>
+    <t>2ARHM</t>
+  </si>
+  <si>
+    <t>2BEM</t>
+  </si>
+  <si>
+    <t>2BLCM</t>
+  </si>
+  <si>
+    <t>4AEM</t>
+  </si>
+  <si>
+    <t>4ALCM</t>
+  </si>
+  <si>
+    <t>4APM</t>
+  </si>
+  <si>
+    <t>4ARHM</t>
+  </si>
+  <si>
+    <t>4BEM</t>
+  </si>
+  <si>
+    <t>4BLCM</t>
+  </si>
+  <si>
+    <t>6AEM</t>
+  </si>
+  <si>
+    <t>6ALCM</t>
+  </si>
+  <si>
+    <t>6APM</t>
+  </si>
+  <si>
+    <t>6ARHM</t>
+  </si>
+  <si>
+    <t>6BEM</t>
+  </si>
+  <si>
+    <t>6BLCM</t>
+  </si>
+  <si>
+    <t>2AEV</t>
+  </si>
+  <si>
+    <t>2ALCV</t>
+  </si>
+  <si>
+    <t>2APV</t>
+  </si>
+  <si>
+    <t>2ARHV</t>
+  </si>
+  <si>
+    <t>2ASV</t>
+  </si>
+  <si>
+    <t>4AEV</t>
+  </si>
+  <si>
+    <t>4ALCV</t>
+  </si>
+  <si>
+    <t>4APV</t>
+  </si>
+  <si>
+    <t>4ARHV</t>
+  </si>
+  <si>
+    <t>4ASV</t>
+  </si>
+  <si>
+    <t>6AEV</t>
+  </si>
+  <si>
+    <t>6ALCV</t>
+  </si>
+  <si>
+    <t>6APV</t>
+  </si>
+  <si>
+    <t>6ARHV</t>
+  </si>
+  <si>
+    <t>6ASV</t>
   </si>
   <si>
     <t>Apro1P</t>
@@ -586,7 +586,7 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -598,236 +598,236 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="G2">
-        <v>9</v>
+        <v>78</v>
       </c>
       <c r="H2">
-        <v>13</v>
+        <v>77</v>
       </c>
       <c r="I2">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="J2">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>154</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>80</v>
+        <v>234</v>
       </c>
       <c r="M2">
-        <v>34.19</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G3">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>79</v>
       </c>
       <c r="I3">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="J3">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="K3">
-        <v>147</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>68</v>
+        <v>209</v>
       </c>
       <c r="M3">
-        <v>31.63</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
       <c r="C4">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="G4">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="H4">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="I4">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="J4">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K4">
-        <v>114</v>
+        <v>29</v>
       </c>
       <c r="L4">
-        <v>72</v>
+        <v>151</v>
       </c>
       <c r="M4">
-        <v>38.71</v>
+        <v>83.89</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
       <c r="C5">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="G5">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="H5">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="I5">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="J5">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K5">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>83</v>
+        <v>172</v>
       </c>
       <c r="M5">
-        <v>43.68</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="G6">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="H6">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="I6">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="K6">
-        <v>103</v>
+        <v>7</v>
       </c>
       <c r="L6">
-        <v>51</v>
+        <v>129</v>
       </c>
       <c r="M6">
-        <v>33.12</v>
+        <v>94.84999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G7">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H7">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="I7">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="J7">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="K7">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="L7">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="M7">
-        <v>52.27</v>
+        <v>84.48</v>
       </c>
     </row>
   </sheetData>
@@ -883,7 +883,7 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -892,239 +892,239 @@
         <v>234</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>195</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>149</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>85</v>
+        <v>234</v>
       </c>
       <c r="M2">
-        <v>36.32</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
         <v>2</v>
       </c>
-      <c r="G3">
-        <v>9</v>
-      </c>
-      <c r="H3">
-        <v>5</v>
-      </c>
       <c r="I3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>134</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>81</v>
+        <v>209</v>
       </c>
       <c r="M3">
-        <v>37.67</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
       <c r="C4">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>180</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>61</v>
+        <v>180</v>
       </c>
       <c r="M4">
-        <v>32.8</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
       <c r="C5">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>136</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="J5">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="K5">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>92</v>
+        <v>172</v>
       </c>
       <c r="M5">
-        <v>48.42</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <v>103</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <v>51</v>
+        <v>136</v>
       </c>
       <c r="M6">
-        <v>33.12</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>112</v>
       </c>
       <c r="F7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H7">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J7">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="M7">
-        <v>46.97</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1180,7 +1180,7 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -1192,236 +1192,236 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="G2">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>77</v>
       </c>
       <c r="I2">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="J2">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>179</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>55</v>
+        <v>234</v>
       </c>
       <c r="M2">
-        <v>23.5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="H3">
-        <v>5</v>
+        <v>79</v>
       </c>
       <c r="I3">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="J3">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="K3">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>46</v>
+        <v>209</v>
       </c>
       <c r="M3">
-        <v>21.4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
       <c r="C4">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="J4">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="K4">
-        <v>152</v>
+        <v>29</v>
       </c>
       <c r="L4">
-        <v>34</v>
+        <v>151</v>
       </c>
       <c r="M4">
-        <v>18.28</v>
+        <v>83.89</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
       <c r="C5">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="I5">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="J5">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="K5">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>58</v>
+        <v>172</v>
       </c>
       <c r="M5">
-        <v>30.53</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="G6">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="I6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="K6">
-        <v>114</v>
+        <v>7</v>
       </c>
       <c r="L6">
-        <v>40</v>
+        <v>129</v>
       </c>
       <c r="M6">
-        <v>25.97</v>
+        <v>94.84999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G7">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H7">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="I7">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="J7">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K7">
-        <v>79</v>
+        <v>18</v>
       </c>
       <c r="L7">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="M7">
-        <v>40.15</v>
+        <v>84.48</v>
       </c>
     </row>
   </sheetData>
@@ -1483,31 +1483,31 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="L2">
-        <v>20.59</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -1515,37 +1515,37 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="L3">
-        <v>26.67</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1553,37 +1553,37 @@
         <v>18</v>
       </c>
       <c r="B4">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="I4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="L4">
-        <v>37.5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1591,37 +1591,37 @@
         <v>19</v>
       </c>
       <c r="B5">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K5">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="L5">
-        <v>11.36</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -1629,7 +1629,7 @@
         <v>20</v>
       </c>
       <c r="B6">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1638,28 +1638,28 @@
         <v>1</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="I6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="L6">
-        <v>20.93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -1667,37 +1667,37 @@
         <v>21</v>
       </c>
       <c r="B7">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F7">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="L7">
-        <v>25.58</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -1705,37 +1705,37 @@
         <v>22</v>
       </c>
       <c r="B8">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G8">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="H8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K8">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="L8">
-        <v>37.5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -1743,37 +1743,37 @@
         <v>23</v>
       </c>
       <c r="B9">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="J9">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K9">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="L9">
-        <v>12.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1781,7 +1781,7 @@
         <v>24</v>
       </c>
       <c r="B10">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -1790,28 +1790,28 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="J10">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="L10">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1819,37 +1819,37 @@
         <v>25</v>
       </c>
       <c r="B11">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11">
         <v>0</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J11">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="K11">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="L11">
-        <v>25.64</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1857,37 +1857,37 @@
         <v>26</v>
       </c>
       <c r="B12">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="H12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J12">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K12">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="L12">
-        <v>35.48</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1895,37 +1895,37 @@
         <v>27</v>
       </c>
       <c r="B13">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="I13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J13">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K13">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="L13">
-        <v>17.78</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1933,37 +1933,37 @@
         <v>28</v>
       </c>
       <c r="B14">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C14">
         <v>0</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I14">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J14">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="K14">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="L14">
-        <v>45.16</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1971,7 +1971,7 @@
         <v>29</v>
       </c>
       <c r="B15">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1989,19 +1989,19 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J15">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L15">
-        <v>11.43</v>
+        <v>14.71</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -2009,37 +2009,37 @@
         <v>30</v>
       </c>
       <c r="B16">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16">
         <v>0</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K16">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="L16">
-        <v>9.52</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -2047,7 +2047,7 @@
         <v>31</v>
       </c>
       <c r="B17">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -2062,22 +2062,22 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="K17">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="L17">
-        <v>5.41</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -2085,37 +2085,37 @@
         <v>32</v>
       </c>
       <c r="B18">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18">
         <v>1</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I18">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K18">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="L18">
-        <v>30</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -2141,19 +2141,19 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I19">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="J19">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="K19">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="L19">
-        <v>9.380000000000001</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -2161,37 +2161,37 @@
         <v>34</v>
       </c>
       <c r="B20">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E20">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20">
+        <v>4</v>
+      </c>
+      <c r="H20">
+        <v>13</v>
+      </c>
+      <c r="I20">
         <v>2</v>
       </c>
-      <c r="H20">
-        <v>4</v>
-      </c>
-      <c r="I20">
-        <v>6</v>
-      </c>
       <c r="J20">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="K20">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="L20">
-        <v>33.33</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -2199,37 +2199,37 @@
         <v>35</v>
       </c>
       <c r="B21">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I21">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J21">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="K21">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="L21">
-        <v>23.53</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -2237,37 +2237,37 @@
         <v>36</v>
       </c>
       <c r="B22">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G22">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H22">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I22">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J22">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="K22">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="L22">
-        <v>34.15</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -2275,7 +2275,7 @@
         <v>37</v>
       </c>
       <c r="B23">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -2293,19 +2293,19 @@
         <v>1</v>
       </c>
       <c r="H23">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="J23">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="K23">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="L23">
-        <v>27.5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -2313,7 +2313,7 @@
         <v>38</v>
       </c>
       <c r="B24">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -2325,25 +2325,25 @@
         <v>0</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H24">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="I24">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J24">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K24">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L24">
-        <v>33.33</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -2351,37 +2351,37 @@
         <v>39</v>
       </c>
       <c r="B25">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E25">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F25">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G25">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="H25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J25">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="K25">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="L25">
-        <v>35</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -2389,37 +2389,37 @@
         <v>40</v>
       </c>
       <c r="B26">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I26">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J26">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K26">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="L26">
-        <v>20.51</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -2427,37 +2427,37 @@
         <v>41</v>
       </c>
       <c r="B27">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D27">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E27">
         <v>1</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H27">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I27">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J27">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K27">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="L27">
-        <v>28.57</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -2465,7 +2465,7 @@
         <v>42</v>
       </c>
       <c r="B28">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -2474,28 +2474,28 @@
         <v>1</v>
       </c>
       <c r="E28">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J28">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="K28">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="L28">
-        <v>18.75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -2503,7 +2503,7 @@
         <v>43</v>
       </c>
       <c r="B29">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -2512,13 +2512,13 @@
         <v>0</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29">
         <v>1</v>
@@ -2527,13 +2527,13 @@
         <v>2</v>
       </c>
       <c r="J29">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="K29">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L29">
-        <v>26.67</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -2541,37 +2541,37 @@
         <v>44</v>
       </c>
       <c r="B30">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C30">
         <v>0</v>
       </c>
       <c r="D30">
+        <v>9</v>
+      </c>
+      <c r="E30">
         <v>2</v>
-      </c>
-      <c r="E30">
-        <v>1</v>
       </c>
       <c r="F30">
         <v>3</v>
       </c>
       <c r="G30">
+        <v>6</v>
+      </c>
+      <c r="H30">
         <v>3</v>
       </c>
-      <c r="H30">
-        <v>7</v>
-      </c>
       <c r="I30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J30">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K30">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="L30">
-        <v>65.38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -2579,37 +2579,37 @@
         <v>45</v>
       </c>
       <c r="B31">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C31">
         <v>0</v>
       </c>
       <c r="D31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G31">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H31">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="I31">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J31">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K31">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="L31">
-        <v>44.44</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -2617,7 +2617,7 @@
         <v>46</v>
       </c>
       <c r="B32">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -2626,28 +2626,28 @@
         <v>0</v>
       </c>
       <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32">
         <v>2</v>
       </c>
-      <c r="F32">
-        <v>0</v>
-      </c>
-      <c r="G32">
-        <v>0</v>
-      </c>
       <c r="H32">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I32">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J32">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="K32">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L32">
-        <v>21.05</v>
+        <v>58.82</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -2655,37 +2655,37 @@
         <v>47</v>
       </c>
       <c r="B33">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C33">
         <v>0</v>
       </c>
       <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33">
         <v>2</v>
       </c>
-      <c r="E33">
-        <v>2</v>
-      </c>
-      <c r="F33">
-        <v>1</v>
-      </c>
       <c r="G33">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H33">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I33">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
         <v>31</v>
       </c>
-      <c r="K33">
-        <v>11</v>
-      </c>
       <c r="L33">
-        <v>26.19</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -2693,7 +2693,7 @@
         <v>48</v>
       </c>
       <c r="B34">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -2708,22 +2708,22 @@
         <v>0</v>
       </c>
       <c r="G34">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H34">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I34">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J34">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K34">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L34">
-        <v>50</v>
+        <v>42.11</v>
       </c>
     </row>
   </sheetData>
@@ -2770,22 +2770,22 @@
         <v>34</v>
       </c>
       <c r="C2">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>61.76</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>55.88</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>79.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2793,25 +2793,25 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>53.33</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>53.33</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>73.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2819,25 +2819,25 @@
         <v>18</v>
       </c>
       <c r="B4">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C4">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>62.5</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>62.5</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>62.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2845,25 +2845,25 @@
         <v>19</v>
       </c>
       <c r="B5">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C5">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>81.81999999999999</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>81.81999999999999</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>88.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2871,25 +2871,25 @@
         <v>20</v>
       </c>
       <c r="B6">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C6">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>62.79</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>53.49</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>79.06999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -2897,25 +2897,25 @@
         <v>21</v>
       </c>
       <c r="B7">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C7">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>67.44</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>69.77</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>74.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2923,25 +2923,25 @@
         <v>22</v>
       </c>
       <c r="B8">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>62.5</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F8">
-        <v>59.38</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>62.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2949,25 +2949,25 @@
         <v>23</v>
       </c>
       <c r="B9">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>68.29000000000001</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>51.22</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>87.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2975,25 +2975,25 @@
         <v>24</v>
       </c>
       <c r="B10">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>88.89</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F10">
-        <v>88.89</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -3001,25 +3001,25 @@
         <v>25</v>
       </c>
       <c r="B11">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>74.36</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>61.54</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>74.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -3027,25 +3027,25 @@
         <v>26</v>
       </c>
       <c r="B12">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C12">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>61.29</v>
+        <v>0</v>
       </c>
       <c r="E12">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>58.06</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>64.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -3053,25 +3053,25 @@
         <v>27</v>
       </c>
       <c r="B13">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C13">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="E13">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>62.22</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>82.22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -3079,25 +3079,25 @@
         <v>28</v>
       </c>
       <c r="B14">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C14">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D14">
-        <v>29.03</v>
+        <v>0</v>
       </c>
       <c r="E14">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>58.06</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>54.84</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -3105,25 +3105,25 @@
         <v>29</v>
       </c>
       <c r="B15">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D15">
-        <v>80</v>
+        <v>85.29000000000001</v>
       </c>
       <c r="E15">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F15">
-        <v>74.29000000000001</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H15">
-        <v>88.56999999999999</v>
+        <v>85.29000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -3131,25 +3131,25 @@
         <v>30</v>
       </c>
       <c r="B16">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>61.9</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>52.38</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>90.48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -3157,25 +3157,25 @@
         <v>31</v>
       </c>
       <c r="B17">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="D17">
-        <v>75.68000000000001</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="F17">
-        <v>75.68000000000001</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H17">
-        <v>94.59</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -3183,25 +3183,25 @@
         <v>32</v>
       </c>
       <c r="B18">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C18">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>46.67</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F18">
-        <v>53.33</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -3212,22 +3212,22 @@
         <v>32</v>
       </c>
       <c r="C19">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D19">
-        <v>68.75</v>
+        <v>0</v>
       </c>
       <c r="E19">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F19">
-        <v>81.25</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="H19">
-        <v>90.63</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -3235,25 +3235,25 @@
         <v>34</v>
       </c>
       <c r="B20">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C20">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="D20">
-        <v>46.15</v>
+        <v>0</v>
       </c>
       <c r="E20">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F20">
-        <v>46.15</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>66.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -3261,25 +3261,25 @@
         <v>35</v>
       </c>
       <c r="B21">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C21">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>64.70999999999999</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F21">
-        <v>61.76</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>76.47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -3287,25 +3287,25 @@
         <v>36</v>
       </c>
       <c r="B22">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C22">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>70.73</v>
+        <v>0</v>
       </c>
       <c r="E22">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F22">
-        <v>60.98</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>65.84999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -3313,25 +3313,25 @@
         <v>37</v>
       </c>
       <c r="B23">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C23">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>57.5</v>
+        <v>0</v>
       </c>
       <c r="E23">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F23">
-        <v>47.5</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="H23">
-        <v>72.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -3339,25 +3339,25 @@
         <v>38</v>
       </c>
       <c r="B24">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C24">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D24">
-        <v>41.67</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F24">
-        <v>41.67</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>66.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -3365,25 +3365,25 @@
         <v>39</v>
       </c>
       <c r="B25">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C25">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="D25">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="E25">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="F25">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="G25">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H25">
-        <v>65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -3391,25 +3391,25 @@
         <v>40</v>
       </c>
       <c r="B26">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C26">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>71.79000000000001</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="F26">
-        <v>74.36</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="H26">
-        <v>79.48999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -3417,25 +3417,25 @@
         <v>41</v>
       </c>
       <c r="B27">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C27">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>60.71</v>
+        <v>0</v>
       </c>
       <c r="E27">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F27">
-        <v>53.57</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>71.43000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -3443,25 +3443,25 @@
         <v>42</v>
       </c>
       <c r="B28">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C28">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>71.88</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F28">
-        <v>78.13</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H28">
-        <v>81.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -3469,25 +3469,25 @@
         <v>43</v>
       </c>
       <c r="B29">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C29">
         <v>7</v>
       </c>
       <c r="D29">
-        <v>46.67</v>
+        <v>50</v>
       </c>
       <c r="E29">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F29">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="G29">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H29">
-        <v>73.33</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -3495,25 +3495,25 @@
         <v>44</v>
       </c>
       <c r="B30">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C30">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D30">
-        <v>34.62</v>
+        <v>0</v>
       </c>
       <c r="E30">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F30">
-        <v>23.08</v>
+        <v>0</v>
       </c>
       <c r="G30">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H30">
-        <v>34.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -3521,25 +3521,25 @@
         <v>45</v>
       </c>
       <c r="B31">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C31">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D31">
-        <v>44.44</v>
+        <v>0</v>
       </c>
       <c r="E31">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F31">
-        <v>51.85</v>
+        <v>0</v>
       </c>
       <c r="G31">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H31">
-        <v>55.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -3547,25 +3547,25 @@
         <v>46</v>
       </c>
       <c r="B32">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C32">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D32">
-        <v>52.63</v>
+        <v>41.18</v>
       </c>
       <c r="E32">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F32">
-        <v>57.89</v>
+        <v>0</v>
       </c>
       <c r="G32">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="H32">
-        <v>78.95</v>
+        <v>41.18</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -3573,25 +3573,25 @@
         <v>47</v>
       </c>
       <c r="B33">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C33">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D33">
-        <v>52.38</v>
+        <v>0</v>
       </c>
       <c r="E33">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="F33">
-        <v>66.67</v>
+        <v>0</v>
       </c>
       <c r="G33">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="H33">
-        <v>73.81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -3599,25 +3599,25 @@
         <v>48</v>
       </c>
       <c r="B34">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C34">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D34">
-        <v>55.56</v>
+        <v>57.89</v>
       </c>
       <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
         <v>11</v>
       </c>
-      <c r="F34">
-        <v>61.11</v>
-      </c>
-      <c r="G34">
-        <v>9</v>
-      </c>
       <c r="H34">
-        <v>50</v>
+        <v>57.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Primer Parcial con Totales
</commit_message>
<xml_diff>
--- a/Totales Generales.xlsx
+++ b/Totales Generales.xlsx
@@ -18,7 +18,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="57">
+  <si>
+    <t>index</t>
+  </si>
   <si>
     <t>Semestre</t>
   </si>
@@ -57,6 +60,9 @@
   </si>
   <si>
     <t>Por_Repro</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
   <si>
     <t>M</t>
@@ -540,10 +546,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -583,251 +589,401 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" t="s">
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2">
+        <v>235</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="H2">
+        <v>7</v>
+      </c>
+      <c r="I2">
         <v>13</v>
       </c>
-      <c r="C2">
-        <v>235</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-      <c r="F2">
+      <c r="J2">
+        <v>20</v>
+      </c>
+      <c r="K2">
+        <v>31</v>
+      </c>
+      <c r="L2">
+        <v>152</v>
+      </c>
+      <c r="M2">
+        <v>83</v>
+      </c>
+      <c r="N2">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3">
+        <v>209</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>7</v>
+      </c>
+      <c r="G3">
+        <v>5</v>
+      </c>
+      <c r="H3">
         <v>8</v>
       </c>
-      <c r="G2">
-        <v>7</v>
-      </c>
-      <c r="H2">
+      <c r="I3">
+        <v>12</v>
+      </c>
+      <c r="J3">
+        <v>14</v>
+      </c>
+      <c r="K3">
+        <v>39</v>
+      </c>
+      <c r="L3">
+        <v>124</v>
+      </c>
+      <c r="M3">
+        <v>85</v>
+      </c>
+      <c r="N3">
+        <v>40.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4">
+        <v>180</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>8</v>
+      </c>
+      <c r="J4">
         <v>13</v>
       </c>
-      <c r="I2">
-        <v>20</v>
-      </c>
-      <c r="J2">
-        <v>31</v>
-      </c>
-      <c r="K2">
-        <v>152</v>
-      </c>
-      <c r="L2">
-        <v>83</v>
-      </c>
-      <c r="M2">
-        <v>35.32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" t="s">
+      <c r="K4">
+        <v>40</v>
+      </c>
+      <c r="L4">
+        <v>117</v>
+      </c>
+      <c r="M4">
+        <v>63</v>
+      </c>
+      <c r="N4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5">
         <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3">
-        <v>209</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>7</v>
-      </c>
-      <c r="F3">
-        <v>5</v>
-      </c>
-      <c r="G3">
-        <v>8</v>
-      </c>
-      <c r="H3">
-        <v>12</v>
-      </c>
-      <c r="I3">
-        <v>14</v>
-      </c>
-      <c r="J3">
-        <v>39</v>
-      </c>
-      <c r="K3">
-        <v>124</v>
-      </c>
-      <c r="L3">
-        <v>85</v>
-      </c>
-      <c r="M3">
-        <v>40.67</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4">
-        <v>180</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>8</v>
-      </c>
-      <c r="I4">
-        <v>13</v>
-      </c>
-      <c r="J4">
-        <v>40</v>
-      </c>
-      <c r="K4">
-        <v>117</v>
-      </c>
-      <c r="L4">
-        <v>63</v>
-      </c>
-      <c r="M4">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" t="s">
-        <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="C5">
-        <v>171</v>
+      <c r="C5" t="s">
+        <v>15</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>624</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F5">
+        <v>11</v>
+      </c>
+      <c r="G5">
         <v>14</v>
-      </c>
-      <c r="G5">
-        <v>10</v>
       </c>
       <c r="H5">
         <v>16</v>
       </c>
       <c r="I5">
+        <v>33</v>
+      </c>
+      <c r="J5">
+        <v>47</v>
+      </c>
+      <c r="K5">
+        <v>110</v>
+      </c>
+      <c r="L5">
+        <v>393</v>
+      </c>
+      <c r="M5">
+        <v>231</v>
+      </c>
+      <c r="N5">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>171</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>14</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6">
+        <v>16</v>
+      </c>
+      <c r="J6">
         <v>27</v>
       </c>
-      <c r="J5">
+      <c r="K6">
         <v>39</v>
       </c>
-      <c r="K5">
+      <c r="L6">
         <v>59</v>
       </c>
-      <c r="L5">
+      <c r="M6">
         <v>112</v>
       </c>
-      <c r="M5">
+      <c r="N6">
         <v>65.5</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
-      <c r="A6" t="s">
+    <row r="7" spans="1:14">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7">
+        <v>138</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
+      <c r="H7">
+        <v>9</v>
+      </c>
+      <c r="I7">
+        <v>13</v>
+      </c>
+      <c r="J7">
+        <v>13</v>
+      </c>
+      <c r="K7">
+        <v>28</v>
+      </c>
+      <c r="L7">
+        <v>56</v>
+      </c>
+      <c r="M7">
+        <v>82</v>
+      </c>
+      <c r="N7">
+        <v>59.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8">
+        <v>116</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
+      </c>
+      <c r="I8">
+        <v>12</v>
+      </c>
+      <c r="J8">
+        <v>15</v>
+      </c>
+      <c r="K8">
+        <v>28</v>
+      </c>
+      <c r="L8">
+        <v>52</v>
+      </c>
+      <c r="M8">
+        <v>64</v>
+      </c>
+      <c r="N8">
+        <v>55.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="C6">
-        <v>138</v>
-      </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6">
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9">
+        <v>425</v>
+      </c>
+      <c r="E9">
+        <v>6</v>
+      </c>
+      <c r="F9">
+        <v>17</v>
+      </c>
+      <c r="G9">
+        <v>20</v>
+      </c>
+      <c r="H9">
+        <v>24</v>
+      </c>
+      <c r="I9">
+        <v>41</v>
+      </c>
+      <c r="J9">
+        <v>55</v>
+      </c>
+      <c r="K9">
+        <v>95</v>
+      </c>
+      <c r="L9">
+        <v>167</v>
+      </c>
+      <c r="M9">
+        <v>258</v>
+      </c>
+      <c r="N9">
+        <v>60.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10">
         <v>8</v>
       </c>
-      <c r="F6">
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10">
+        <v>1049</v>
+      </c>
+      <c r="E10">
         <v>6</v>
       </c>
-      <c r="G6">
-        <v>9</v>
-      </c>
-      <c r="H6">
-        <v>13</v>
-      </c>
-      <c r="I6">
-        <v>13</v>
-      </c>
-      <c r="J6">
+      <c r="F10">
         <v>28</v>
       </c>
-      <c r="K6">
-        <v>56</v>
-      </c>
-      <c r="L6">
-        <v>82</v>
-      </c>
-      <c r="M6">
-        <v>59.42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7">
-        <v>116</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>4</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>5</v>
-      </c>
-      <c r="H7">
-        <v>12</v>
-      </c>
-      <c r="I7">
-        <v>15</v>
-      </c>
-      <c r="J7">
-        <v>28</v>
-      </c>
-      <c r="K7">
-        <v>52</v>
-      </c>
-      <c r="L7">
-        <v>64</v>
-      </c>
-      <c r="M7">
-        <v>55.17</v>
+      <c r="G10">
+        <v>34</v>
+      </c>
+      <c r="H10">
+        <v>40</v>
+      </c>
+      <c r="I10">
+        <v>74</v>
+      </c>
+      <c r="J10">
+        <v>102</v>
+      </c>
+      <c r="K10">
+        <v>205</v>
+      </c>
+      <c r="L10">
+        <v>560</v>
+      </c>
+      <c r="M10">
+        <v>489</v>
+      </c>
+      <c r="N10">
+        <v>46.6</v>
       </c>
     </row>
   </sheetData>
@@ -837,10 +993,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -880,26 +1036,29 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" t="s">
-        <v>8</v>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2">
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2">
         <v>235</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>39</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>196</v>
       </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
       <c r="G2">
         <v>0</v>
       </c>
@@ -916,194 +1075,209 @@
         <v>0</v>
       </c>
       <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
         <v>235</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
-      <c r="A3" t="s">
+    <row r="3" spans="1:14">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3">
+        <v>209</v>
+      </c>
+      <c r="E3">
+        <v>168</v>
+      </c>
+      <c r="F3">
+        <v>38</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>209</v>
+      </c>
+      <c r="N3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4">
+        <v>180</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>180</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>180</v>
+      </c>
+      <c r="N4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5">
         <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3">
-        <v>209</v>
-      </c>
-      <c r="D3">
-        <v>168</v>
-      </c>
-      <c r="E3">
-        <v>38</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
-        <v>209</v>
-      </c>
-      <c r="M3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4">
-        <v>180</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>180</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
-        <v>180</v>
-      </c>
-      <c r="M4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" t="s">
-        <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5">
+        <v>624</v>
+      </c>
+      <c r="E5">
+        <v>207</v>
+      </c>
+      <c r="F5">
+        <v>414</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>624</v>
+      </c>
+      <c r="N5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6">
         <v>171</v>
       </c>
-      <c r="D5">
+      <c r="E6">
         <v>30</v>
       </c>
-      <c r="E5">
+      <c r="F6">
         <v>135</v>
       </c>
-      <c r="F5">
+      <c r="G6">
         <v>2</v>
       </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
         <v>3</v>
       </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
         <v>171</v>
       </c>
-      <c r="M5">
+      <c r="N6">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6">
+    <row r="7" spans="1:14">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7">
         <v>138</v>
       </c>
-      <c r="D6">
+      <c r="E7">
         <v>88</v>
       </c>
-      <c r="E6">
+      <c r="F7">
         <v>46</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>138</v>
-      </c>
-      <c r="M6">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7">
-        <v>116</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>112</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -1121,9 +1295,141 @@
         <v>0</v>
       </c>
       <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>138</v>
+      </c>
+      <c r="N7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8">
         <v>116</v>
       </c>
-      <c r="M7">
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>112</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>2</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>116</v>
+      </c>
+      <c r="N8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9">
+        <v>425</v>
+      </c>
+      <c r="E9">
+        <v>118</v>
+      </c>
+      <c r="F9">
+        <v>293</v>
+      </c>
+      <c r="G9">
+        <v>3</v>
+      </c>
+      <c r="H9">
+        <v>2</v>
+      </c>
+      <c r="I9">
+        <v>4</v>
+      </c>
+      <c r="J9">
+        <v>5</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>425</v>
+      </c>
+      <c r="N9">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10">
+        <v>1049</v>
+      </c>
+      <c r="E10">
+        <v>325</v>
+      </c>
+      <c r="F10">
+        <v>707</v>
+      </c>
+      <c r="G10">
+        <v>3</v>
+      </c>
+      <c r="H10">
+        <v>3</v>
+      </c>
+      <c r="I10">
+        <v>6</v>
+      </c>
+      <c r="J10">
+        <v>5</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>1049</v>
+      </c>
+      <c r="N10">
         <v>100</v>
       </c>
     </row>
@@ -1134,10 +1440,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1177,251 +1483,401 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" t="s">
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2">
+        <v>235</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="H2">
+        <v>7</v>
+      </c>
+      <c r="I2">
         <v>13</v>
       </c>
-      <c r="C2">
-        <v>235</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-      <c r="F2">
+      <c r="J2">
+        <v>20</v>
+      </c>
+      <c r="K2">
+        <v>31</v>
+      </c>
+      <c r="L2">
+        <v>152</v>
+      </c>
+      <c r="M2">
+        <v>83</v>
+      </c>
+      <c r="N2">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3">
+        <v>209</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>7</v>
+      </c>
+      <c r="G3">
+        <v>5</v>
+      </c>
+      <c r="H3">
         <v>8</v>
       </c>
-      <c r="G2">
-        <v>7</v>
-      </c>
-      <c r="H2">
+      <c r="I3">
+        <v>12</v>
+      </c>
+      <c r="J3">
+        <v>14</v>
+      </c>
+      <c r="K3">
+        <v>39</v>
+      </c>
+      <c r="L3">
+        <v>124</v>
+      </c>
+      <c r="M3">
+        <v>85</v>
+      </c>
+      <c r="N3">
+        <v>40.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4">
+        <v>180</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>8</v>
+      </c>
+      <c r="J4">
         <v>13</v>
       </c>
-      <c r="I2">
-        <v>20</v>
-      </c>
-      <c r="J2">
-        <v>31</v>
-      </c>
-      <c r="K2">
-        <v>152</v>
-      </c>
-      <c r="L2">
-        <v>83</v>
-      </c>
-      <c r="M2">
-        <v>35.32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" t="s">
+      <c r="K4">
+        <v>40</v>
+      </c>
+      <c r="L4">
+        <v>117</v>
+      </c>
+      <c r="M4">
+        <v>63</v>
+      </c>
+      <c r="N4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5">
         <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3">
-        <v>209</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>7</v>
-      </c>
-      <c r="F3">
-        <v>5</v>
-      </c>
-      <c r="G3">
-        <v>8</v>
-      </c>
-      <c r="H3">
-        <v>12</v>
-      </c>
-      <c r="I3">
-        <v>14</v>
-      </c>
-      <c r="J3">
-        <v>39</v>
-      </c>
-      <c r="K3">
-        <v>124</v>
-      </c>
-      <c r="L3">
-        <v>85</v>
-      </c>
-      <c r="M3">
-        <v>40.67</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4">
-        <v>180</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>8</v>
-      </c>
-      <c r="I4">
-        <v>13</v>
-      </c>
-      <c r="J4">
-        <v>40</v>
-      </c>
-      <c r="K4">
-        <v>117</v>
-      </c>
-      <c r="L4">
-        <v>63</v>
-      </c>
-      <c r="M4">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" t="s">
-        <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="C5">
-        <v>171</v>
+      <c r="C5" t="s">
+        <v>15</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>624</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F5">
+        <v>11</v>
+      </c>
+      <c r="G5">
         <v>14</v>
-      </c>
-      <c r="G5">
-        <v>10</v>
       </c>
       <c r="H5">
         <v>16</v>
       </c>
       <c r="I5">
+        <v>33</v>
+      </c>
+      <c r="J5">
+        <v>47</v>
+      </c>
+      <c r="K5">
+        <v>110</v>
+      </c>
+      <c r="L5">
+        <v>393</v>
+      </c>
+      <c r="M5">
+        <v>231</v>
+      </c>
+      <c r="N5">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>171</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>14</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6">
+        <v>16</v>
+      </c>
+      <c r="J6">
         <v>27</v>
       </c>
-      <c r="J5">
+      <c r="K6">
         <v>39</v>
       </c>
-      <c r="K5">
+      <c r="L6">
         <v>59</v>
       </c>
-      <c r="L5">
+      <c r="M6">
         <v>112</v>
       </c>
-      <c r="M5">
+      <c r="N6">
         <v>65.5</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
-      <c r="A6" t="s">
+    <row r="7" spans="1:14">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7">
+        <v>138</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
+      <c r="H7">
+        <v>9</v>
+      </c>
+      <c r="I7">
+        <v>13</v>
+      </c>
+      <c r="J7">
+        <v>13</v>
+      </c>
+      <c r="K7">
+        <v>28</v>
+      </c>
+      <c r="L7">
+        <v>56</v>
+      </c>
+      <c r="M7">
+        <v>82</v>
+      </c>
+      <c r="N7">
+        <v>59.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8">
+        <v>116</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
+      </c>
+      <c r="I8">
+        <v>12</v>
+      </c>
+      <c r="J8">
+        <v>15</v>
+      </c>
+      <c r="K8">
+        <v>28</v>
+      </c>
+      <c r="L8">
+        <v>52</v>
+      </c>
+      <c r="M8">
+        <v>64</v>
+      </c>
+      <c r="N8">
+        <v>55.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="C6">
-        <v>138</v>
-      </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6">
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9">
+        <v>425</v>
+      </c>
+      <c r="E9">
+        <v>6</v>
+      </c>
+      <c r="F9">
+        <v>17</v>
+      </c>
+      <c r="G9">
+        <v>20</v>
+      </c>
+      <c r="H9">
+        <v>24</v>
+      </c>
+      <c r="I9">
+        <v>41</v>
+      </c>
+      <c r="J9">
+        <v>55</v>
+      </c>
+      <c r="K9">
+        <v>95</v>
+      </c>
+      <c r="L9">
+        <v>167</v>
+      </c>
+      <c r="M9">
+        <v>258</v>
+      </c>
+      <c r="N9">
+        <v>60.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10">
         <v>8</v>
       </c>
-      <c r="F6">
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10">
+        <v>1049</v>
+      </c>
+      <c r="E10">
         <v>6</v>
       </c>
-      <c r="G6">
-        <v>9</v>
-      </c>
-      <c r="H6">
-        <v>13</v>
-      </c>
-      <c r="I6">
-        <v>13</v>
-      </c>
-      <c r="J6">
+      <c r="F10">
         <v>28</v>
       </c>
-      <c r="K6">
-        <v>56</v>
-      </c>
-      <c r="L6">
-        <v>82</v>
-      </c>
-      <c r="M6">
-        <v>59.42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7">
-        <v>116</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>4</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>5</v>
-      </c>
-      <c r="H7">
-        <v>12</v>
-      </c>
-      <c r="I7">
-        <v>15</v>
-      </c>
-      <c r="J7">
-        <v>28</v>
-      </c>
-      <c r="K7">
-        <v>52</v>
-      </c>
-      <c r="L7">
-        <v>64</v>
-      </c>
-      <c r="M7">
-        <v>55.17</v>
+      <c r="G10">
+        <v>34</v>
+      </c>
+      <c r="H10">
+        <v>40</v>
+      </c>
+      <c r="I10">
+        <v>74</v>
+      </c>
+      <c r="J10">
+        <v>102</v>
+      </c>
+      <c r="K10">
+        <v>205</v>
+      </c>
+      <c r="L10">
+        <v>560</v>
+      </c>
+      <c r="M10">
+        <v>489</v>
+      </c>
+      <c r="N10">
+        <v>46.6</v>
       </c>
     </row>
   </sheetData>
@@ -1436,45 +1892,45 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>34</v>
@@ -1512,7 +1968,7 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B3">
         <v>43</v>
@@ -1550,7 +2006,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B4">
         <v>39</v>
@@ -1588,7 +2044,7 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B5">
         <v>40</v>
@@ -1626,7 +2082,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>37</v>
@@ -1664,7 +2120,7 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B7">
         <v>42</v>
@@ -1702,7 +2158,7 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B8">
         <v>31</v>
@@ -1740,7 +2196,7 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B9">
         <v>42</v>
@@ -1778,7 +2234,7 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B10">
         <v>28</v>
@@ -1816,7 +2272,7 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B11">
         <v>38</v>
@@ -1854,7 +2310,7 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B12">
         <v>29</v>
@@ -1892,7 +2348,7 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B13">
         <v>41</v>
@@ -1930,7 +2386,7 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B14">
         <v>30</v>
@@ -1968,7 +2424,7 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B15">
         <v>34</v>
@@ -2006,7 +2462,7 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B16">
         <v>20</v>
@@ -2044,7 +2500,7 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B17">
         <v>36</v>
@@ -2082,7 +2538,7 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B18">
         <v>28</v>
@@ -2120,7 +2576,7 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B19">
         <v>32</v>
@@ -2158,7 +2614,7 @@
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B20">
         <v>33</v>
@@ -2196,7 +2652,7 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B21">
         <v>42</v>
@@ -2234,7 +2690,7 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B22">
         <v>30</v>
@@ -2272,7 +2728,7 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B23">
         <v>33</v>
@@ -2310,7 +2766,7 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B24">
         <v>33</v>
@@ -2348,7 +2804,7 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B25">
         <v>33</v>
@@ -2386,7 +2842,7 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B26">
         <v>36</v>
@@ -2424,7 +2880,7 @@
     </row>
     <row r="27" spans="1:12">
       <c r="A27" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B27">
         <v>25</v>
@@ -2462,7 +2918,7 @@
     </row>
     <row r="28" spans="1:12">
       <c r="A28" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B28">
         <v>30</v>
@@ -2500,7 +2956,7 @@
     </row>
     <row r="29" spans="1:12">
       <c r="A29" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B29">
         <v>14</v>
@@ -2538,7 +2994,7 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B30">
         <v>23</v>
@@ -2576,7 +3032,7 @@
     </row>
     <row r="31" spans="1:12">
       <c r="A31" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B31">
         <v>26</v>
@@ -2614,7 +3070,7 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B32">
         <v>17</v>
@@ -2652,7 +3108,7 @@
     </row>
     <row r="33" spans="1:12">
       <c r="A33" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B33">
         <v>31</v>
@@ -2690,7 +3146,7 @@
     </row>
     <row r="34" spans="1:12">
       <c r="A34" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B34">
         <v>19</v>
@@ -2738,33 +3194,33 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>34</v>
@@ -2790,7 +3246,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B3">
         <v>43</v>
@@ -2816,7 +3272,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B4">
         <v>39</v>
@@ -2842,7 +3298,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B5">
         <v>40</v>
@@ -2868,7 +3324,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>37</v>
@@ -2894,7 +3350,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B7">
         <v>42</v>
@@ -2920,7 +3376,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B8">
         <v>31</v>
@@ -2946,7 +3402,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B9">
         <v>42</v>
@@ -2972,7 +3428,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B10">
         <v>28</v>
@@ -2998,7 +3454,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B11">
         <v>38</v>
@@ -3024,7 +3480,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B12">
         <v>29</v>
@@ -3050,7 +3506,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B13">
         <v>41</v>
@@ -3076,7 +3532,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B14">
         <v>30</v>
@@ -3102,7 +3558,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B15">
         <v>34</v>
@@ -3128,7 +3584,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B16">
         <v>20</v>
@@ -3154,7 +3610,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B17">
         <v>36</v>
@@ -3180,7 +3636,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B18">
         <v>28</v>
@@ -3206,7 +3662,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B19">
         <v>32</v>
@@ -3232,7 +3688,7 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B20">
         <v>33</v>
@@ -3258,7 +3714,7 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B21">
         <v>42</v>
@@ -3284,7 +3740,7 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B22">
         <v>30</v>
@@ -3310,7 +3766,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B23">
         <v>33</v>
@@ -3336,7 +3792,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B24">
         <v>33</v>
@@ -3362,7 +3818,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B25">
         <v>33</v>
@@ -3388,7 +3844,7 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B26">
         <v>36</v>
@@ -3414,7 +3870,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B27">
         <v>25</v>
@@ -3440,7 +3896,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B28">
         <v>30</v>
@@ -3466,7 +3922,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B29">
         <v>14</v>
@@ -3492,7 +3948,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B30">
         <v>23</v>
@@ -3518,7 +3974,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B31">
         <v>26</v>
@@ -3544,7 +4000,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B32">
         <v>17</v>
@@ -3570,7 +4026,7 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B33">
         <v>31</v>
@@ -3596,7 +4052,7 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B34">
         <v>19</v>

</xml_diff>

<commit_message>
Primer Parcial Totales Corregidos
</commit_message>
<xml_diff>
--- a/Totales Generales.xlsx
+++ b/Totales Generales.xlsx
@@ -18,10 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="57">
-  <si>
-    <t>index</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="56">
   <si>
     <t>Semestre</t>
   </si>
@@ -546,10 +543,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -589,400 +586,370 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>235</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2">
-        <v>235</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
+      <c r="I2">
+        <v>20</v>
+      </c>
+      <c r="J2">
+        <v>31</v>
+      </c>
+      <c r="K2">
+        <v>152</v>
+      </c>
+      <c r="L2">
+        <v>83</v>
+      </c>
+      <c r="M2">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
+        <v>209</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>8</v>
+      </c>
+      <c r="H3">
+        <v>12</v>
+      </c>
+      <c r="I3">
+        <v>14</v>
+      </c>
+      <c r="J3">
+        <v>39</v>
+      </c>
+      <c r="K3">
+        <v>124</v>
+      </c>
+      <c r="L3">
+        <v>85</v>
+      </c>
+      <c r="M3">
+        <v>40.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="G2">
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>180</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
         <v>8</v>
       </c>
-      <c r="H2">
-        <v>7</v>
-      </c>
-      <c r="I2">
+      <c r="I4">
         <v>13</v>
       </c>
-      <c r="J2">
-        <v>20</v>
-      </c>
-      <c r="K2">
-        <v>31</v>
-      </c>
-      <c r="L2">
-        <v>152</v>
-      </c>
-      <c r="M2">
-        <v>83</v>
-      </c>
-      <c r="N2">
-        <v>35.3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3">
-        <v>209</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>7</v>
-      </c>
-      <c r="G3">
-        <v>5</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>12</v>
-      </c>
-      <c r="J3">
-        <v>14</v>
-      </c>
-      <c r="K3">
-        <v>39</v>
-      </c>
-      <c r="L3">
-        <v>124</v>
-      </c>
-      <c r="M3">
-        <v>85</v>
-      </c>
-      <c r="N3">
-        <v>40.7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4">
-        <v>180</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>8</v>
-      </c>
       <c r="J4">
+        <v>40</v>
+      </c>
+      <c r="K4">
+        <v>117</v>
+      </c>
+      <c r="L4">
+        <v>63</v>
+      </c>
+      <c r="M4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" t="s">
         <v>13</v>
-      </c>
-      <c r="K4">
-        <v>40</v>
-      </c>
-      <c r="L4">
-        <v>117</v>
-      </c>
-      <c r="M4">
-        <v>63</v>
-      </c>
-      <c r="N4">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="A5">
-        <v>6</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5">
+        <v>624</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>11</v>
+      </c>
+      <c r="F5">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>16</v>
+      </c>
+      <c r="H5">
+        <v>33</v>
+      </c>
+      <c r="I5">
+        <v>47</v>
+      </c>
+      <c r="J5">
+        <v>110</v>
+      </c>
+      <c r="K5">
+        <v>393</v>
+      </c>
+      <c r="L5">
+        <v>231</v>
+      </c>
+      <c r="M5">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="D5">
-        <v>624</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>11</v>
-      </c>
-      <c r="G5">
+      <c r="C6">
+        <v>171</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
         <v>14</v>
       </c>
-      <c r="H5">
+      <c r="G6">
+        <v>10</v>
+      </c>
+      <c r="H6">
         <v>16</v>
       </c>
-      <c r="I5">
-        <v>33</v>
-      </c>
-      <c r="J5">
-        <v>47</v>
-      </c>
-      <c r="K5">
-        <v>110</v>
-      </c>
-      <c r="L5">
-        <v>393</v>
-      </c>
-      <c r="M5">
-        <v>231</v>
-      </c>
-      <c r="N5">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="I6">
+        <v>27</v>
+      </c>
+      <c r="J6">
+        <v>39</v>
+      </c>
+      <c r="K6">
+        <v>59</v>
+      </c>
+      <c r="L6">
+        <v>112</v>
+      </c>
+      <c r="M6">
+        <v>65.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7">
+        <v>138</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>8</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="G7">
         <v>9</v>
       </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>171</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>5</v>
-      </c>
-      <c r="G6">
-        <v>14</v>
-      </c>
-      <c r="H6">
-        <v>10</v>
-      </c>
-      <c r="I6">
-        <v>16</v>
-      </c>
-      <c r="J6">
-        <v>27</v>
-      </c>
-      <c r="K6">
-        <v>39</v>
-      </c>
-      <c r="L6">
-        <v>59</v>
-      </c>
-      <c r="M6">
-        <v>112</v>
-      </c>
-      <c r="N6">
-        <v>65.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7">
-        <v>138</v>
-      </c>
-      <c r="E7">
-        <v>5</v>
-      </c>
-      <c r="F7">
-        <v>8</v>
-      </c>
-      <c r="G7">
-        <v>6</v>
-      </c>
       <c r="H7">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I7">
         <v>13</v>
       </c>
       <c r="J7">
+        <v>28</v>
+      </c>
+      <c r="K7">
+        <v>56</v>
+      </c>
+      <c r="L7">
+        <v>82</v>
+      </c>
+      <c r="M7">
+        <v>59.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <v>116</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>4</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>5</v>
+      </c>
+      <c r="H8">
+        <v>12</v>
+      </c>
+      <c r="I8">
+        <v>15</v>
+      </c>
+      <c r="J8">
+        <v>28</v>
+      </c>
+      <c r="K8">
+        <v>52</v>
+      </c>
+      <c r="L8">
+        <v>64</v>
+      </c>
+      <c r="M8">
+        <v>55.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" t="s">
         <v>13</v>
       </c>
-      <c r="K7">
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>425</v>
+      </c>
+      <c r="D9">
+        <v>6</v>
+      </c>
+      <c r="E9">
+        <v>17</v>
+      </c>
+      <c r="F9">
+        <v>20</v>
+      </c>
+      <c r="G9">
+        <v>24</v>
+      </c>
+      <c r="H9">
+        <v>41</v>
+      </c>
+      <c r="I9">
+        <v>55</v>
+      </c>
+      <c r="J9">
+        <v>95</v>
+      </c>
+      <c r="K9">
+        <v>167</v>
+      </c>
+      <c r="L9">
+        <v>258</v>
+      </c>
+      <c r="M9">
+        <v>60.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10">
+        <v>1049</v>
+      </c>
+      <c r="D10">
+        <v>6</v>
+      </c>
+      <c r="E10">
         <v>28</v>
       </c>
-      <c r="L7">
-        <v>56</v>
-      </c>
-      <c r="M7">
-        <v>82</v>
-      </c>
-      <c r="N7">
-        <v>59.4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8">
-        <v>116</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>4</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>5</v>
-      </c>
-      <c r="I8">
-        <v>12</v>
-      </c>
-      <c r="J8">
-        <v>15</v>
-      </c>
-      <c r="K8">
-        <v>28</v>
-      </c>
-      <c r="L8">
-        <v>52</v>
-      </c>
-      <c r="M8">
-        <v>64</v>
-      </c>
-      <c r="N8">
-        <v>55.2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9">
-        <v>425</v>
-      </c>
-      <c r="E9">
-        <v>6</v>
-      </c>
-      <c r="F9">
-        <v>17</v>
-      </c>
-      <c r="G9">
-        <v>20</v>
-      </c>
-      <c r="H9">
-        <v>24</v>
-      </c>
-      <c r="I9">
-        <v>41</v>
-      </c>
-      <c r="J9">
-        <v>55</v>
-      </c>
-      <c r="K9">
-        <v>95</v>
-      </c>
-      <c r="L9">
-        <v>167</v>
-      </c>
-      <c r="M9">
-        <v>258</v>
-      </c>
-      <c r="N9">
-        <v>60.7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10">
-        <v>1049</v>
-      </c>
-      <c r="E10">
-        <v>6</v>
-      </c>
       <c r="F10">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G10">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H10">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="I10">
-        <v>74</v>
+        <v>102</v>
       </c>
       <c r="J10">
-        <v>102</v>
+        <v>205</v>
       </c>
       <c r="K10">
-        <v>205</v>
+        <v>560</v>
       </c>
       <c r="L10">
-        <v>560</v>
+        <v>489</v>
       </c>
       <c r="M10">
-        <v>489</v>
-      </c>
-      <c r="N10">
         <v>46.6</v>
       </c>
     </row>
@@ -993,10 +960,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1036,400 +1003,370 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>235</v>
+      </c>
+      <c r="D2">
+        <v>39</v>
+      </c>
+      <c r="E2">
+        <v>196</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>235</v>
+      </c>
+      <c r="M2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
+        <v>209</v>
+      </c>
+      <c r="D3">
+        <v>168</v>
+      </c>
+      <c r="E3">
+        <v>38</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>209</v>
+      </c>
+      <c r="M3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>180</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>180</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>180</v>
+      </c>
+      <c r="M4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2">
-        <v>235</v>
-      </c>
-      <c r="E2">
-        <v>39</v>
-      </c>
-      <c r="F2">
-        <v>196</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>235</v>
-      </c>
-      <c r="N2">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3">
-        <v>209</v>
-      </c>
-      <c r="E3">
-        <v>168</v>
-      </c>
-      <c r="F3">
-        <v>38</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>209</v>
-      </c>
-      <c r="N3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4">
-        <v>180</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>180</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>180</v>
-      </c>
-      <c r="N4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="A5">
-        <v>6</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5">
+        <v>624</v>
+      </c>
+      <c r="D5">
+        <v>207</v>
+      </c>
+      <c r="E5">
+        <v>414</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>624</v>
+      </c>
+      <c r="M5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="D5">
-        <v>624</v>
-      </c>
-      <c r="E5">
-        <v>207</v>
-      </c>
-      <c r="F5">
-        <v>414</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
+      <c r="C6">
+        <v>171</v>
+      </c>
+      <c r="D6">
+        <v>30</v>
+      </c>
+      <c r="E6">
+        <v>135</v>
+      </c>
+      <c r="F6">
         <v>2</v>
       </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>624</v>
-      </c>
-      <c r="N5">
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>3</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>171</v>
+      </c>
+      <c r="M6">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
-      <c r="A6">
+    <row r="7" spans="1:13">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7">
+        <v>138</v>
+      </c>
+      <c r="D7">
+        <v>88</v>
+      </c>
+      <c r="E7">
+        <v>46</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>138</v>
+      </c>
+      <c r="M7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <v>116</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>112</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>116</v>
+      </c>
+      <c r="M8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>425</v>
+      </c>
+      <c r="D9">
+        <v>118</v>
+      </c>
+      <c r="E9">
+        <v>293</v>
+      </c>
+      <c r="F9">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>171</v>
-      </c>
-      <c r="E6">
-        <v>30</v>
-      </c>
-      <c r="F6">
-        <v>135</v>
-      </c>
-      <c r="G6">
+      <c r="G9">
         <v>2</v>
       </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6">
+      <c r="H9">
+        <v>4</v>
+      </c>
+      <c r="I9">
+        <v>5</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>425</v>
+      </c>
+      <c r="M9">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10">
+        <v>1049</v>
+      </c>
+      <c r="D10">
+        <v>325</v>
+      </c>
+      <c r="E10">
+        <v>707</v>
+      </c>
+      <c r="F10">
         <v>3</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>171</v>
-      </c>
-      <c r="N6">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7">
-        <v>138</v>
-      </c>
-      <c r="E7">
-        <v>88</v>
-      </c>
-      <c r="F7">
-        <v>46</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>2</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>138</v>
-      </c>
-      <c r="N7">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8">
-        <v>116</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>112</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>1</v>
-      </c>
-      <c r="I8">
-        <v>1</v>
-      </c>
-      <c r="J8">
-        <v>2</v>
-      </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>116</v>
-      </c>
-      <c r="N8">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9">
-        <v>425</v>
-      </c>
-      <c r="E9">
-        <v>118</v>
-      </c>
-      <c r="F9">
-        <v>293</v>
-      </c>
-      <c r="G9">
-        <v>3</v>
-      </c>
-      <c r="H9">
-        <v>2</v>
-      </c>
-      <c r="I9">
-        <v>4</v>
-      </c>
-      <c r="J9">
-        <v>5</v>
-      </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9">
-        <v>425</v>
-      </c>
-      <c r="N9">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10">
-        <v>1049</v>
-      </c>
-      <c r="E10">
-        <v>325</v>
-      </c>
-      <c r="F10">
-        <v>707</v>
       </c>
       <c r="G10">
         <v>3</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J10">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>0</v>
+        <v>1049</v>
       </c>
       <c r="M10">
-        <v>1049</v>
-      </c>
-      <c r="N10">
         <v>100</v>
       </c>
     </row>
@@ -1440,10 +1377,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1483,400 +1420,370 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>235</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2">
-        <v>235</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
+      <c r="I2">
+        <v>20</v>
+      </c>
+      <c r="J2">
+        <v>31</v>
+      </c>
+      <c r="K2">
+        <v>152</v>
+      </c>
+      <c r="L2">
+        <v>83</v>
+      </c>
+      <c r="M2">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
+        <v>209</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>8</v>
+      </c>
+      <c r="H3">
+        <v>12</v>
+      </c>
+      <c r="I3">
+        <v>14</v>
+      </c>
+      <c r="J3">
+        <v>39</v>
+      </c>
+      <c r="K3">
+        <v>124</v>
+      </c>
+      <c r="L3">
+        <v>85</v>
+      </c>
+      <c r="M3">
+        <v>40.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="G2">
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>180</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
         <v>8</v>
       </c>
-      <c r="H2">
-        <v>7</v>
-      </c>
-      <c r="I2">
+      <c r="I4">
         <v>13</v>
       </c>
-      <c r="J2">
-        <v>20</v>
-      </c>
-      <c r="K2">
-        <v>31</v>
-      </c>
-      <c r="L2">
-        <v>152</v>
-      </c>
-      <c r="M2">
-        <v>83</v>
-      </c>
-      <c r="N2">
-        <v>35.3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3">
-        <v>209</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>7</v>
-      </c>
-      <c r="G3">
-        <v>5</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>12</v>
-      </c>
-      <c r="J3">
-        <v>14</v>
-      </c>
-      <c r="K3">
-        <v>39</v>
-      </c>
-      <c r="L3">
-        <v>124</v>
-      </c>
-      <c r="M3">
-        <v>85</v>
-      </c>
-      <c r="N3">
-        <v>40.7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4">
-        <v>180</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>8</v>
-      </c>
       <c r="J4">
+        <v>40</v>
+      </c>
+      <c r="K4">
+        <v>117</v>
+      </c>
+      <c r="L4">
+        <v>63</v>
+      </c>
+      <c r="M4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" t="s">
         <v>13</v>
-      </c>
-      <c r="K4">
-        <v>40</v>
-      </c>
-      <c r="L4">
-        <v>117</v>
-      </c>
-      <c r="M4">
-        <v>63</v>
-      </c>
-      <c r="N4">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="A5">
-        <v>6</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5">
+        <v>624</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>11</v>
+      </c>
+      <c r="F5">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>16</v>
+      </c>
+      <c r="H5">
+        <v>33</v>
+      </c>
+      <c r="I5">
+        <v>47</v>
+      </c>
+      <c r="J5">
+        <v>110</v>
+      </c>
+      <c r="K5">
+        <v>393</v>
+      </c>
+      <c r="L5">
+        <v>231</v>
+      </c>
+      <c r="M5">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="D5">
-        <v>624</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>11</v>
-      </c>
-      <c r="G5">
+      <c r="C6">
+        <v>171</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
         <v>14</v>
       </c>
-      <c r="H5">
+      <c r="G6">
+        <v>10</v>
+      </c>
+      <c r="H6">
         <v>16</v>
       </c>
-      <c r="I5">
-        <v>33</v>
-      </c>
-      <c r="J5">
-        <v>47</v>
-      </c>
-      <c r="K5">
-        <v>110</v>
-      </c>
-      <c r="L5">
-        <v>393</v>
-      </c>
-      <c r="M5">
-        <v>231</v>
-      </c>
-      <c r="N5">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="I6">
+        <v>27</v>
+      </c>
+      <c r="J6">
+        <v>39</v>
+      </c>
+      <c r="K6">
+        <v>59</v>
+      </c>
+      <c r="L6">
+        <v>112</v>
+      </c>
+      <c r="M6">
+        <v>65.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7">
+        <v>138</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>8</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="G7">
         <v>9</v>
       </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>171</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>5</v>
-      </c>
-      <c r="G6">
-        <v>14</v>
-      </c>
-      <c r="H6">
-        <v>10</v>
-      </c>
-      <c r="I6">
-        <v>16</v>
-      </c>
-      <c r="J6">
-        <v>27</v>
-      </c>
-      <c r="K6">
-        <v>39</v>
-      </c>
-      <c r="L6">
-        <v>59</v>
-      </c>
-      <c r="M6">
-        <v>112</v>
-      </c>
-      <c r="N6">
-        <v>65.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7">
-        <v>138</v>
-      </c>
-      <c r="E7">
-        <v>5</v>
-      </c>
-      <c r="F7">
-        <v>8</v>
-      </c>
-      <c r="G7">
-        <v>6</v>
-      </c>
       <c r="H7">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I7">
         <v>13</v>
       </c>
       <c r="J7">
+        <v>28</v>
+      </c>
+      <c r="K7">
+        <v>56</v>
+      </c>
+      <c r="L7">
+        <v>82</v>
+      </c>
+      <c r="M7">
+        <v>59.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <v>116</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>4</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>5</v>
+      </c>
+      <c r="H8">
+        <v>12</v>
+      </c>
+      <c r="I8">
+        <v>15</v>
+      </c>
+      <c r="J8">
+        <v>28</v>
+      </c>
+      <c r="K8">
+        <v>52</v>
+      </c>
+      <c r="L8">
+        <v>64</v>
+      </c>
+      <c r="M8">
+        <v>55.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" t="s">
         <v>13</v>
       </c>
-      <c r="K7">
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>425</v>
+      </c>
+      <c r="D9">
+        <v>6</v>
+      </c>
+      <c r="E9">
+        <v>17</v>
+      </c>
+      <c r="F9">
+        <v>20</v>
+      </c>
+      <c r="G9">
+        <v>24</v>
+      </c>
+      <c r="H9">
+        <v>41</v>
+      </c>
+      <c r="I9">
+        <v>55</v>
+      </c>
+      <c r="J9">
+        <v>95</v>
+      </c>
+      <c r="K9">
+        <v>167</v>
+      </c>
+      <c r="L9">
+        <v>258</v>
+      </c>
+      <c r="M9">
+        <v>60.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10">
+        <v>1049</v>
+      </c>
+      <c r="D10">
+        <v>6</v>
+      </c>
+      <c r="E10">
         <v>28</v>
       </c>
-      <c r="L7">
-        <v>56</v>
-      </c>
-      <c r="M7">
-        <v>82</v>
-      </c>
-      <c r="N7">
-        <v>59.4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8">
-        <v>116</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>4</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>5</v>
-      </c>
-      <c r="I8">
-        <v>12</v>
-      </c>
-      <c r="J8">
-        <v>15</v>
-      </c>
-      <c r="K8">
-        <v>28</v>
-      </c>
-      <c r="L8">
-        <v>52</v>
-      </c>
-      <c r="M8">
-        <v>64</v>
-      </c>
-      <c r="N8">
-        <v>55.2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9">
-        <v>425</v>
-      </c>
-      <c r="E9">
-        <v>6</v>
-      </c>
-      <c r="F9">
-        <v>17</v>
-      </c>
-      <c r="G9">
-        <v>20</v>
-      </c>
-      <c r="H9">
-        <v>24</v>
-      </c>
-      <c r="I9">
-        <v>41</v>
-      </c>
-      <c r="J9">
-        <v>55</v>
-      </c>
-      <c r="K9">
-        <v>95</v>
-      </c>
-      <c r="L9">
-        <v>167</v>
-      </c>
-      <c r="M9">
-        <v>258</v>
-      </c>
-      <c r="N9">
-        <v>60.7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10">
-        <v>1049</v>
-      </c>
-      <c r="E10">
-        <v>6</v>
-      </c>
       <c r="F10">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G10">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H10">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="I10">
-        <v>74</v>
+        <v>102</v>
       </c>
       <c r="J10">
-        <v>102</v>
+        <v>205</v>
       </c>
       <c r="K10">
-        <v>205</v>
+        <v>560</v>
       </c>
       <c r="L10">
-        <v>560</v>
+        <v>489</v>
       </c>
       <c r="M10">
-        <v>489</v>
-      </c>
-      <c r="N10">
         <v>46.6</v>
       </c>
     </row>
@@ -1892,45 +1799,45 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2">
         <v>34</v>
@@ -1968,7 +1875,7 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3">
         <v>43</v>
@@ -2006,7 +1913,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4">
         <v>39</v>
@@ -2044,7 +1951,7 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5">
         <v>40</v>
@@ -2082,7 +1989,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6">
         <v>37</v>
@@ -2120,7 +2027,7 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7">
         <v>42</v>
@@ -2158,7 +2065,7 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B8">
         <v>31</v>
@@ -2196,7 +2103,7 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B9">
         <v>42</v>
@@ -2234,7 +2141,7 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10">
         <v>28</v>
@@ -2272,7 +2179,7 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B11">
         <v>38</v>
@@ -2310,7 +2217,7 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12">
         <v>29</v>
@@ -2348,7 +2255,7 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13">
         <v>41</v>
@@ -2386,7 +2293,7 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14">
         <v>30</v>
@@ -2424,7 +2331,7 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15">
         <v>34</v>
@@ -2462,7 +2369,7 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16">
         <v>20</v>
@@ -2500,7 +2407,7 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B17">
         <v>36</v>
@@ -2538,7 +2445,7 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B18">
         <v>28</v>
@@ -2576,7 +2483,7 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B19">
         <v>32</v>
@@ -2614,7 +2521,7 @@
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B20">
         <v>33</v>
@@ -2652,7 +2559,7 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B21">
         <v>42</v>
@@ -2690,7 +2597,7 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B22">
         <v>30</v>
@@ -2728,7 +2635,7 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B23">
         <v>33</v>
@@ -2766,7 +2673,7 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B24">
         <v>33</v>
@@ -2804,7 +2711,7 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B25">
         <v>33</v>
@@ -2842,7 +2749,7 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B26">
         <v>36</v>
@@ -2880,7 +2787,7 @@
     </row>
     <row r="27" spans="1:12">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B27">
         <v>25</v>
@@ -2918,7 +2825,7 @@
     </row>
     <row r="28" spans="1:12">
       <c r="A28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B28">
         <v>30</v>
@@ -2956,7 +2863,7 @@
     </row>
     <row r="29" spans="1:12">
       <c r="A29" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B29">
         <v>14</v>
@@ -2994,7 +2901,7 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B30">
         <v>23</v>
@@ -3032,7 +2939,7 @@
     </row>
     <row r="31" spans="1:12">
       <c r="A31" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B31">
         <v>26</v>
@@ -3070,7 +2977,7 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32">
         <v>17</v>
@@ -3108,7 +3015,7 @@
     </row>
     <row r="33" spans="1:12">
       <c r="A33" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B33">
         <v>31</v>
@@ -3146,7 +3053,7 @@
     </row>
     <row r="34" spans="1:12">
       <c r="A34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B34">
         <v>19</v>
@@ -3194,33 +3101,33 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2">
         <v>34</v>
@@ -3246,7 +3153,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3">
         <v>43</v>
@@ -3272,7 +3179,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4">
         <v>39</v>
@@ -3298,7 +3205,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5">
         <v>40</v>
@@ -3324,7 +3231,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6">
         <v>37</v>
@@ -3350,7 +3257,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7">
         <v>42</v>
@@ -3376,7 +3283,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B8">
         <v>31</v>
@@ -3402,7 +3309,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B9">
         <v>42</v>
@@ -3428,7 +3335,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10">
         <v>28</v>
@@ -3454,7 +3361,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B11">
         <v>38</v>
@@ -3480,7 +3387,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12">
         <v>29</v>
@@ -3506,7 +3413,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13">
         <v>41</v>
@@ -3532,7 +3439,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14">
         <v>30</v>
@@ -3558,7 +3465,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15">
         <v>34</v>
@@ -3584,7 +3491,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16">
         <v>20</v>
@@ -3610,7 +3517,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B17">
         <v>36</v>
@@ -3636,7 +3543,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B18">
         <v>28</v>
@@ -3662,7 +3569,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B19">
         <v>32</v>
@@ -3688,7 +3595,7 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B20">
         <v>33</v>
@@ -3714,7 +3621,7 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B21">
         <v>42</v>
@@ -3740,7 +3647,7 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B22">
         <v>30</v>
@@ -3766,7 +3673,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B23">
         <v>33</v>
@@ -3792,7 +3699,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B24">
         <v>33</v>
@@ -3818,7 +3725,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B25">
         <v>33</v>
@@ -3844,7 +3751,7 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B26">
         <v>36</v>
@@ -3870,7 +3777,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B27">
         <v>25</v>
@@ -3896,7 +3803,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B28">
         <v>30</v>
@@ -3922,7 +3829,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B29">
         <v>14</v>
@@ -3948,7 +3855,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B30">
         <v>23</v>
@@ -3974,7 +3881,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B31">
         <v>26</v>
@@ -4000,7 +3907,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32">
         <v>17</v>
@@ -4026,7 +3933,7 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B33">
         <v>31</v>
@@ -4052,7 +3959,7 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B34">
         <v>19</v>

</xml_diff>

<commit_message>
cambio en el código y de formato
</commit_message>
<xml_diff>
--- a/Totales Generales.xlsx
+++ b/Totales Generales.xlsx
@@ -173,16 +173,16 @@
     <t>Apro1P</t>
   </si>
   <si>
+    <t>Apro2P</t>
+  </si>
+  <si>
+    <t>AproFin</t>
+  </si>
+  <si>
     <t>Por_Apro1P</t>
   </si>
   <si>
-    <t>Apro2P</t>
-  </si>
-  <si>
     <t>Por_Apro2P</t>
-  </si>
-  <si>
-    <t>AproFin</t>
   </si>
   <si>
     <t>Por_AproFin</t>
@@ -192,6 +192,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0\%"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -244,8 +247,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -545,45 +549,48 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="13" max="13" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -624,7 +631,7 @@
       <c r="L2">
         <v>83</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="1">
         <v>35.3</v>
       </c>
     </row>
@@ -665,7 +672,7 @@
       <c r="L3">
         <v>85</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="1">
         <v>40.7</v>
       </c>
     </row>
@@ -706,7 +713,7 @@
       <c r="L4">
         <v>63</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="1">
         <v>35</v>
       </c>
     </row>
@@ -747,7 +754,7 @@
       <c r="L5">
         <v>231</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="1">
         <v>37</v>
       </c>
     </row>
@@ -788,7 +795,7 @@
       <c r="L6">
         <v>112</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="1">
         <v>65.5</v>
       </c>
     </row>
@@ -829,7 +836,7 @@
       <c r="L7">
         <v>82</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="1">
         <v>59.4</v>
       </c>
     </row>
@@ -870,7 +877,7 @@
       <c r="L8">
         <v>64</v>
       </c>
-      <c r="M8">
+      <c r="M8" s="1">
         <v>55.2</v>
       </c>
     </row>
@@ -911,7 +918,7 @@
       <c r="L9">
         <v>258</v>
       </c>
-      <c r="M9">
+      <c r="M9" s="1">
         <v>60.7</v>
       </c>
     </row>
@@ -949,7 +956,7 @@
       <c r="L10">
         <v>489</v>
       </c>
-      <c r="M10">
+      <c r="M10" s="1">
         <v>46.6</v>
       </c>
     </row>
@@ -962,45 +969,48 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="13" max="13" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1041,7 +1051,7 @@
       <c r="L2">
         <v>235</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="1">
         <v>100</v>
       </c>
     </row>
@@ -1082,7 +1092,7 @@
       <c r="L3">
         <v>209</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="1">
         <v>100</v>
       </c>
     </row>
@@ -1123,7 +1133,7 @@
       <c r="L4">
         <v>180</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="1">
         <v>100</v>
       </c>
     </row>
@@ -1164,7 +1174,7 @@
       <c r="L5">
         <v>624</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="1">
         <v>100</v>
       </c>
     </row>
@@ -1205,7 +1215,7 @@
       <c r="L6">
         <v>171</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="1">
         <v>100</v>
       </c>
     </row>
@@ -1246,7 +1256,7 @@
       <c r="L7">
         <v>138</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="1">
         <v>100</v>
       </c>
     </row>
@@ -1287,7 +1297,7 @@
       <c r="L8">
         <v>116</v>
       </c>
-      <c r="M8">
+      <c r="M8" s="1">
         <v>100</v>
       </c>
     </row>
@@ -1328,7 +1338,7 @@
       <c r="L9">
         <v>425</v>
       </c>
-      <c r="M9">
+      <c r="M9" s="1">
         <v>100</v>
       </c>
     </row>
@@ -1366,7 +1376,7 @@
       <c r="L10">
         <v>1049</v>
       </c>
-      <c r="M10">
+      <c r="M10" s="1">
         <v>100</v>
       </c>
     </row>
@@ -1379,45 +1389,48 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="13" max="13" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1458,7 +1471,7 @@
       <c r="L2">
         <v>83</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="1">
         <v>35.3</v>
       </c>
     </row>
@@ -1499,7 +1512,7 @@
       <c r="L3">
         <v>85</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="1">
         <v>40.7</v>
       </c>
     </row>
@@ -1540,7 +1553,7 @@
       <c r="L4">
         <v>63</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="1">
         <v>35</v>
       </c>
     </row>
@@ -1581,7 +1594,7 @@
       <c r="L5">
         <v>231</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="1">
         <v>37</v>
       </c>
     </row>
@@ -1622,7 +1635,7 @@
       <c r="L6">
         <v>112</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="1">
         <v>65.5</v>
       </c>
     </row>
@@ -1663,7 +1676,7 @@
       <c r="L7">
         <v>82</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="1">
         <v>59.4</v>
       </c>
     </row>
@@ -1704,7 +1717,7 @@
       <c r="L8">
         <v>64</v>
       </c>
-      <c r="M8">
+      <c r="M8" s="1">
         <v>55.2</v>
       </c>
     </row>
@@ -1745,7 +1758,7 @@
       <c r="L9">
         <v>258</v>
       </c>
-      <c r="M9">
+      <c r="M9" s="1">
         <v>60.7</v>
       </c>
     </row>
@@ -1783,7 +1796,7 @@
       <c r="L10">
         <v>489</v>
       </c>
-      <c r="M10">
+      <c r="M10" s="1">
         <v>46.6</v>
       </c>
     </row>
@@ -1796,42 +1809,45 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L34"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="12" max="12" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1869,8 +1885,8 @@
       <c r="K2">
         <v>11</v>
       </c>
-      <c r="L2">
-        <v>32.35</v>
+      <c r="L2" s="1">
+        <v>32.4</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -1907,8 +1923,8 @@
       <c r="K3">
         <v>10</v>
       </c>
-      <c r="L3">
-        <v>23.26</v>
+      <c r="L3" s="1">
+        <v>23.3</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1945,8 +1961,8 @@
       <c r="K4">
         <v>19</v>
       </c>
-      <c r="L4">
-        <v>48.72</v>
+      <c r="L4" s="1">
+        <v>48.7</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1983,7 +1999,7 @@
       <c r="K5">
         <v>9</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="1">
         <v>22.5</v>
       </c>
     </row>
@@ -2021,8 +2037,8 @@
       <c r="K6">
         <v>17</v>
       </c>
-      <c r="L6">
-        <v>45.95</v>
+      <c r="L6" s="1">
+        <v>45.9</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -2059,8 +2075,8 @@
       <c r="K7">
         <v>17</v>
       </c>
-      <c r="L7">
-        <v>40.48</v>
+      <c r="L7" s="1">
+        <v>40.5</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2097,8 +2113,8 @@
       <c r="K8">
         <v>14</v>
       </c>
-      <c r="L8">
-        <v>45.16</v>
+      <c r="L8" s="1">
+        <v>45.2</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2135,8 +2151,8 @@
       <c r="K9">
         <v>11</v>
       </c>
-      <c r="L9">
-        <v>26.19</v>
+      <c r="L9" s="1">
+        <v>26.2</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -2173,8 +2189,8 @@
       <c r="K10">
         <v>11</v>
       </c>
-      <c r="L10">
-        <v>39.29</v>
+      <c r="L10" s="1">
+        <v>39.3</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -2211,8 +2227,8 @@
       <c r="K11">
         <v>13</v>
       </c>
-      <c r="L11">
-        <v>34.21</v>
+      <c r="L11" s="1">
+        <v>34.2</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -2249,8 +2265,8 @@
       <c r="K12">
         <v>15</v>
       </c>
-      <c r="L12">
-        <v>51.72</v>
+      <c r="L12" s="1">
+        <v>51.7</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -2287,8 +2303,8 @@
       <c r="K13">
         <v>21</v>
       </c>
-      <c r="L13">
-        <v>51.22</v>
+      <c r="L13" s="1">
+        <v>51.2</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -2325,8 +2341,8 @@
       <c r="K14">
         <v>16</v>
       </c>
-      <c r="L14">
-        <v>53.33</v>
+      <c r="L14" s="1">
+        <v>53.3</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -2363,8 +2379,8 @@
       <c r="K15">
         <v>5</v>
       </c>
-      <c r="L15">
-        <v>14.71</v>
+      <c r="L15" s="1">
+        <v>14.7</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -2401,7 +2417,7 @@
       <c r="K16">
         <v>14</v>
       </c>
-      <c r="L16">
+      <c r="L16" s="1">
         <v>70</v>
       </c>
     </row>
@@ -2439,8 +2455,8 @@
       <c r="K17">
         <v>6</v>
       </c>
-      <c r="L17">
-        <v>16.67</v>
+      <c r="L17" s="1">
+        <v>16.7</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -2477,8 +2493,8 @@
       <c r="K18">
         <v>19</v>
       </c>
-      <c r="L18">
-        <v>67.86</v>
+      <c r="L18" s="1">
+        <v>67.90000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -2515,8 +2531,8 @@
       <c r="K19">
         <v>3</v>
       </c>
-      <c r="L19">
-        <v>9.380000000000001</v>
+      <c r="L19" s="1">
+        <v>9.4</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -2553,8 +2569,8 @@
       <c r="K20">
         <v>28</v>
       </c>
-      <c r="L20">
-        <v>84.84999999999999</v>
+      <c r="L20" s="1">
+        <v>84.8</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -2591,8 +2607,8 @@
       <c r="K21">
         <v>27</v>
       </c>
-      <c r="L21">
-        <v>64.29000000000001</v>
+      <c r="L21" s="1">
+        <v>64.3</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -2629,7 +2645,7 @@
       <c r="K22">
         <v>27</v>
       </c>
-      <c r="L22">
+      <c r="L22" s="1">
         <v>90</v>
       </c>
     </row>
@@ -2667,8 +2683,8 @@
       <c r="K23">
         <v>11</v>
       </c>
-      <c r="L23">
-        <v>33.33</v>
+      <c r="L23" s="1">
+        <v>33.3</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -2705,8 +2721,8 @@
       <c r="K24">
         <v>19</v>
       </c>
-      <c r="L24">
-        <v>57.58</v>
+      <c r="L24" s="1">
+        <v>57.6</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -2743,8 +2759,8 @@
       <c r="K25">
         <v>19</v>
       </c>
-      <c r="L25">
-        <v>57.58</v>
+      <c r="L25" s="1">
+        <v>57.6</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -2781,8 +2797,8 @@
       <c r="K26">
         <v>21</v>
       </c>
-      <c r="L26">
-        <v>58.33</v>
+      <c r="L26" s="1">
+        <v>58.3</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -2819,7 +2835,7 @@
       <c r="K27">
         <v>18</v>
       </c>
-      <c r="L27">
+      <c r="L27" s="1">
         <v>72</v>
       </c>
     </row>
@@ -2857,7 +2873,7 @@
       <c r="K28">
         <v>18</v>
       </c>
-      <c r="L28">
+      <c r="L28" s="1">
         <v>60</v>
       </c>
     </row>
@@ -2895,8 +2911,8 @@
       <c r="K29">
         <v>6</v>
       </c>
-      <c r="L29">
-        <v>42.86</v>
+      <c r="L29" s="1">
+        <v>42.9</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -2933,8 +2949,8 @@
       <c r="K30">
         <v>16</v>
       </c>
-      <c r="L30">
-        <v>69.56999999999999</v>
+      <c r="L30" s="1">
+        <v>69.59999999999999</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -2971,8 +2987,8 @@
       <c r="K31">
         <v>14</v>
       </c>
-      <c r="L31">
-        <v>53.85</v>
+      <c r="L31" s="1">
+        <v>53.8</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -3009,8 +3025,8 @@
       <c r="K32">
         <v>10</v>
       </c>
-      <c r="L32">
-        <v>58.82</v>
+      <c r="L32" s="1">
+        <v>58.8</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -3047,8 +3063,8 @@
       <c r="K33">
         <v>16</v>
       </c>
-      <c r="L33">
-        <v>51.61</v>
+      <c r="L33" s="1">
+        <v>51.6</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -3085,8 +3101,8 @@
       <c r="K34">
         <v>8</v>
       </c>
-      <c r="L34">
-        <v>42.11</v>
+      <c r="L34" s="1">
+        <v>42.1</v>
       </c>
     </row>
   </sheetData>
@@ -3098,30 +3114,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="6" max="8" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>55</v>
       </c>
     </row>
@@ -3136,19 +3155,19 @@
         <v>23</v>
       </c>
       <c r="D2">
-        <v>67.65000000000001</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
         <v>23</v>
       </c>
-      <c r="H2">
-        <v>67.65000000000001</v>
+      <c r="F2" s="1">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>67.59999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -3162,19 +3181,19 @@
         <v>33</v>
       </c>
       <c r="D3">
-        <v>76.73999999999999</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
         <v>33</v>
       </c>
-      <c r="H3">
-        <v>76.73999999999999</v>
+      <c r="F3" s="1">
+        <v>76.7</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>76.7</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -3188,19 +3207,19 @@
         <v>20</v>
       </c>
       <c r="D4">
-        <v>51.28</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
         <v>20</v>
       </c>
-      <c r="H4">
-        <v>51.28</v>
+      <c r="F4" s="1">
+        <v>51.3</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1">
+        <v>51.3</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -3214,18 +3233,18 @@
         <v>31</v>
       </c>
       <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>31</v>
+      </c>
+      <c r="F5" s="1">
         <v>77.5</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>31</v>
-      </c>
-      <c r="H5">
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
         <v>77.5</v>
       </c>
     </row>
@@ -3240,19 +3259,19 @@
         <v>20</v>
       </c>
       <c r="D6">
-        <v>54.05</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
         <v>20</v>
       </c>
-      <c r="H6">
-        <v>54.05</v>
+      <c r="F6" s="1">
+        <v>54.1</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0</v>
+      </c>
+      <c r="H6" s="1">
+        <v>54.1</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -3266,19 +3285,19 @@
         <v>25</v>
       </c>
       <c r="D7">
-        <v>59.52</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
         <v>25</v>
       </c>
-      <c r="H7">
-        <v>59.52</v>
+      <c r="F7" s="1">
+        <v>59.5</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1">
+        <v>59.5</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -3292,19 +3311,19 @@
         <v>17</v>
       </c>
       <c r="D8">
-        <v>54.84</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
         <v>17</v>
       </c>
-      <c r="H8">
-        <v>54.84</v>
+      <c r="F8" s="1">
+        <v>54.8</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1">
+        <v>54.8</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3318,19 +3337,19 @@
         <v>31</v>
       </c>
       <c r="D9">
-        <v>73.81</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
         <v>31</v>
       </c>
-      <c r="H9">
-        <v>73.81</v>
+      <c r="F9" s="1">
+        <v>73.8</v>
+      </c>
+      <c r="G9" s="1">
+        <v>0</v>
+      </c>
+      <c r="H9" s="1">
+        <v>73.8</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -3344,19 +3363,19 @@
         <v>17</v>
       </c>
       <c r="D10">
-        <v>60.71</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10">
         <v>17</v>
       </c>
-      <c r="H10">
-        <v>60.71</v>
+      <c r="F10" s="1">
+        <v>60.7</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0</v>
+      </c>
+      <c r="H10" s="1">
+        <v>60.7</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -3370,19 +3389,19 @@
         <v>25</v>
       </c>
       <c r="D11">
-        <v>65.79000000000001</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11">
         <v>25</v>
       </c>
-      <c r="H11">
-        <v>65.79000000000001</v>
+      <c r="F11" s="1">
+        <v>65.8</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0</v>
+      </c>
+      <c r="H11" s="1">
+        <v>65.8</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -3396,19 +3415,19 @@
         <v>14</v>
       </c>
       <c r="D12">
-        <v>48.28</v>
+        <v>0</v>
       </c>
       <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12">
         <v>14</v>
       </c>
-      <c r="H12">
-        <v>48.28</v>
+      <c r="F12" s="1">
+        <v>48.3</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>48.3</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -3422,19 +3441,19 @@
         <v>20</v>
       </c>
       <c r="D13">
-        <v>48.78</v>
+        <v>0</v>
       </c>
       <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13">
         <v>20</v>
       </c>
-      <c r="H13">
-        <v>48.78</v>
+      <c r="F13" s="1">
+        <v>48.8</v>
+      </c>
+      <c r="G13" s="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>48.8</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -3448,19 +3467,19 @@
         <v>14</v>
       </c>
       <c r="D14">
-        <v>46.67</v>
+        <v>0</v>
       </c>
       <c r="E14">
-        <v>0</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14">
         <v>14</v>
       </c>
-      <c r="H14">
-        <v>46.67</v>
+      <c r="F14" s="1">
+        <v>46.7</v>
+      </c>
+      <c r="G14" s="1">
+        <v>0</v>
+      </c>
+      <c r="H14" s="1">
+        <v>46.7</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -3474,19 +3493,19 @@
         <v>29</v>
       </c>
       <c r="D15">
-        <v>85.29000000000001</v>
+        <v>0</v>
       </c>
       <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15">
         <v>29</v>
       </c>
-      <c r="H15">
-        <v>85.29000000000001</v>
+      <c r="F15" s="1">
+        <v>85.3</v>
+      </c>
+      <c r="G15" s="1">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
+        <v>85.3</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -3500,18 +3519,18 @@
         <v>6</v>
       </c>
       <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>6</v>
+      </c>
+      <c r="F16" s="1">
         <v>30</v>
       </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-      <c r="G16">
-        <v>6</v>
-      </c>
-      <c r="H16">
+      <c r="G16" s="1">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
         <v>30</v>
       </c>
     </row>
@@ -3526,19 +3545,19 @@
         <v>30</v>
       </c>
       <c r="D17">
-        <v>83.33</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>0</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-      <c r="G17">
         <v>30</v>
       </c>
-      <c r="H17">
-        <v>83.33</v>
+      <c r="F17" s="1">
+        <v>83.3</v>
+      </c>
+      <c r="G17" s="1">
+        <v>0</v>
+      </c>
+      <c r="H17" s="1">
+        <v>83.3</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -3552,19 +3571,19 @@
         <v>9</v>
       </c>
       <c r="D18">
-        <v>32.14</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>0</v>
-      </c>
-      <c r="F18">
-        <v>0</v>
-      </c>
-      <c r="G18">
         <v>9</v>
       </c>
-      <c r="H18">
-        <v>32.14</v>
+      <c r="F18" s="1">
+        <v>32.1</v>
+      </c>
+      <c r="G18" s="1">
+        <v>0</v>
+      </c>
+      <c r="H18" s="1">
+        <v>32.1</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -3578,19 +3597,19 @@
         <v>29</v>
       </c>
       <c r="D19">
-        <v>90.63</v>
+        <v>0</v>
       </c>
       <c r="E19">
-        <v>0</v>
-      </c>
-      <c r="F19">
-        <v>0</v>
-      </c>
-      <c r="G19">
         <v>29</v>
       </c>
-      <c r="H19">
-        <v>90.63</v>
+      <c r="F19" s="1">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="G19" s="1">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>90.59999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -3604,19 +3623,19 @@
         <v>5</v>
       </c>
       <c r="D20">
-        <v>15.15</v>
+        <v>0</v>
       </c>
       <c r="E20">
-        <v>0</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-      <c r="G20">
         <v>5</v>
       </c>
-      <c r="H20">
-        <v>15.15</v>
+      <c r="F20" s="1">
+        <v>15.2</v>
+      </c>
+      <c r="G20" s="1">
+        <v>0</v>
+      </c>
+      <c r="H20" s="1">
+        <v>15.2</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -3630,19 +3649,19 @@
         <v>15</v>
       </c>
       <c r="D21">
-        <v>35.71</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>0</v>
-      </c>
-      <c r="F21">
-        <v>0</v>
-      </c>
-      <c r="G21">
         <v>15</v>
       </c>
-      <c r="H21">
-        <v>35.71</v>
+      <c r="F21" s="1">
+        <v>35.7</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0</v>
+      </c>
+      <c r="H21" s="1">
+        <v>35.7</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -3656,18 +3675,18 @@
         <v>3</v>
       </c>
       <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>3</v>
+      </c>
+      <c r="F22" s="1">
         <v>10</v>
       </c>
-      <c r="E22">
-        <v>0</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-      <c r="G22">
-        <v>3</v>
-      </c>
-      <c r="H22">
+      <c r="G22" s="1">
+        <v>0</v>
+      </c>
+      <c r="H22" s="1">
         <v>10</v>
       </c>
     </row>
@@ -3682,19 +3701,19 @@
         <v>22</v>
       </c>
       <c r="D23">
-        <v>66.67</v>
+        <v>0</v>
       </c>
       <c r="E23">
-        <v>0</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-      <c r="G23">
         <v>22</v>
       </c>
-      <c r="H23">
-        <v>66.67</v>
+      <c r="F23" s="1">
+        <v>66.7</v>
+      </c>
+      <c r="G23" s="1">
+        <v>0</v>
+      </c>
+      <c r="H23" s="1">
+        <v>66.7</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -3708,19 +3727,19 @@
         <v>14</v>
       </c>
       <c r="D24">
-        <v>42.42</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>0</v>
-      </c>
-      <c r="F24">
-        <v>0</v>
-      </c>
-      <c r="G24">
         <v>14</v>
       </c>
-      <c r="H24">
-        <v>42.42</v>
+      <c r="F24" s="1">
+        <v>42.4</v>
+      </c>
+      <c r="G24" s="1">
+        <v>0</v>
+      </c>
+      <c r="H24" s="1">
+        <v>42.4</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -3734,19 +3753,19 @@
         <v>14</v>
       </c>
       <c r="D25">
-        <v>42.42</v>
+        <v>0</v>
       </c>
       <c r="E25">
-        <v>0</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-      <c r="G25">
         <v>14</v>
       </c>
-      <c r="H25">
-        <v>42.42</v>
+      <c r="F25" s="1">
+        <v>42.4</v>
+      </c>
+      <c r="G25" s="1">
+        <v>0</v>
+      </c>
+      <c r="H25" s="1">
+        <v>42.4</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -3760,19 +3779,19 @@
         <v>15</v>
       </c>
       <c r="D26">
-        <v>41.67</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>0</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-      <c r="G26">
         <v>15</v>
       </c>
-      <c r="H26">
-        <v>41.67</v>
+      <c r="F26" s="1">
+        <v>41.7</v>
+      </c>
+      <c r="G26" s="1">
+        <v>0</v>
+      </c>
+      <c r="H26" s="1">
+        <v>41.7</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -3786,18 +3805,18 @@
         <v>7</v>
       </c>
       <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>7</v>
+      </c>
+      <c r="F27" s="1">
         <v>28</v>
       </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
-      <c r="G27">
-        <v>7</v>
-      </c>
-      <c r="H27">
+      <c r="G27" s="1">
+        <v>0</v>
+      </c>
+      <c r="H27" s="1">
         <v>28</v>
       </c>
     </row>
@@ -3812,18 +3831,18 @@
         <v>12</v>
       </c>
       <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>12</v>
+      </c>
+      <c r="F28" s="1">
         <v>40</v>
       </c>
-      <c r="E28">
-        <v>0</v>
-      </c>
-      <c r="F28">
-        <v>0</v>
-      </c>
-      <c r="G28">
-        <v>12</v>
-      </c>
-      <c r="H28">
+      <c r="G28" s="1">
+        <v>0</v>
+      </c>
+      <c r="H28" s="1">
         <v>40</v>
       </c>
     </row>
@@ -3838,19 +3857,19 @@
         <v>8</v>
       </c>
       <c r="D29">
-        <v>57.14</v>
+        <v>0</v>
       </c>
       <c r="E29">
-        <v>0</v>
-      </c>
-      <c r="F29">
-        <v>0</v>
-      </c>
-      <c r="G29">
         <v>8</v>
       </c>
-      <c r="H29">
-        <v>57.14</v>
+      <c r="F29" s="1">
+        <v>57.1</v>
+      </c>
+      <c r="G29" s="1">
+        <v>0</v>
+      </c>
+      <c r="H29" s="1">
+        <v>57.1</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -3864,19 +3883,19 @@
         <v>7</v>
       </c>
       <c r="D30">
-        <v>30.43</v>
+        <v>0</v>
       </c>
       <c r="E30">
-        <v>0</v>
-      </c>
-      <c r="F30">
-        <v>0</v>
-      </c>
-      <c r="G30">
         <v>7</v>
       </c>
-      <c r="H30">
-        <v>30.43</v>
+      <c r="F30" s="1">
+        <v>30.4</v>
+      </c>
+      <c r="G30" s="1">
+        <v>0</v>
+      </c>
+      <c r="H30" s="1">
+        <v>30.4</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -3890,19 +3909,19 @@
         <v>12</v>
       </c>
       <c r="D31">
-        <v>46.15</v>
+        <v>0</v>
       </c>
       <c r="E31">
-        <v>0</v>
-      </c>
-      <c r="F31">
-        <v>0</v>
-      </c>
-      <c r="G31">
         <v>12</v>
       </c>
-      <c r="H31">
-        <v>46.15</v>
+      <c r="F31" s="1">
+        <v>46.2</v>
+      </c>
+      <c r="G31" s="1">
+        <v>0</v>
+      </c>
+      <c r="H31" s="1">
+        <v>46.2</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -3916,19 +3935,19 @@
         <v>7</v>
       </c>
       <c r="D32">
-        <v>41.18</v>
+        <v>0</v>
       </c>
       <c r="E32">
-        <v>0</v>
-      </c>
-      <c r="F32">
-        <v>0</v>
-      </c>
-      <c r="G32">
         <v>7</v>
       </c>
-      <c r="H32">
-        <v>41.18</v>
+      <c r="F32" s="1">
+        <v>41.2</v>
+      </c>
+      <c r="G32" s="1">
+        <v>0</v>
+      </c>
+      <c r="H32" s="1">
+        <v>41.2</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -3942,19 +3961,19 @@
         <v>15</v>
       </c>
       <c r="D33">
-        <v>48.39</v>
+        <v>0</v>
       </c>
       <c r="E33">
-        <v>0</v>
-      </c>
-      <c r="F33">
-        <v>0</v>
-      </c>
-      <c r="G33">
         <v>15</v>
       </c>
-      <c r="H33">
-        <v>48.39</v>
+      <c r="F33" s="1">
+        <v>48.4</v>
+      </c>
+      <c r="G33" s="1">
+        <v>0</v>
+      </c>
+      <c r="H33" s="1">
+        <v>48.4</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -3968,19 +3987,19 @@
         <v>11</v>
       </c>
       <c r="D34">
-        <v>57.89</v>
+        <v>0</v>
       </c>
       <c r="E34">
-        <v>0</v>
-      </c>
-      <c r="F34">
-        <v>0</v>
-      </c>
-      <c r="G34">
         <v>11</v>
       </c>
-      <c r="H34">
-        <v>57.89</v>
+      <c r="F34" s="1">
+        <v>57.9</v>
+      </c>
+      <c r="G34" s="1">
+        <v>0</v>
+      </c>
+      <c r="H34" s="1">
+        <v>57.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Segundo Parcial 16 mayo
</commit_message>
<xml_diff>
--- a/Totales Generales.xlsx
+++ b/Totales Generales.xlsx
@@ -617,22 +617,22 @@
         <v>7</v>
       </c>
       <c r="H2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J2">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="L2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="M2" s="1">
-        <v>35.3</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -658,10 +658,10 @@
         <v>8</v>
       </c>
       <c r="H3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I3">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J3">
         <v>39</v>
@@ -746,16 +746,16 @@
         <v>47</v>
       </c>
       <c r="J5">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K5">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="L5">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="M5" s="1">
-        <v>37</v>
+        <v>36.9</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -766,7 +766,7 @@
         <v>15</v>
       </c>
       <c r="C6">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -775,7 +775,7 @@
         <v>5</v>
       </c>
       <c r="F6">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G6">
         <v>10</v>
@@ -793,10 +793,10 @@
         <v>59</v>
       </c>
       <c r="L6">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="M6" s="1">
-        <v>65.5</v>
+        <v>65.7</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -810,13 +810,13 @@
         <v>138</v>
       </c>
       <c r="D7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E7">
         <v>8</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G7">
         <v>9</v>
@@ -889,16 +889,16 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E9">
         <v>17</v>
       </c>
       <c r="F9">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G9">
         <v>24</v>
@@ -916,10 +916,10 @@
         <v>167</v>
       </c>
       <c r="L9">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="M9" s="1">
-        <v>60.7</v>
+        <v>60.8</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -927,16 +927,16 @@
         <v>13</v>
       </c>
       <c r="C10">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="D10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E10">
         <v>28</v>
       </c>
       <c r="F10">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G10">
         <v>40</v>
@@ -948,10 +948,10 @@
         <v>102</v>
       </c>
       <c r="J10">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K10">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="L10">
         <v>489</v>
@@ -1025,16 +1025,16 @@
         <v>235</v>
       </c>
       <c r="D2">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>196</v>
+        <v>43</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -1066,34 +1066,34 @@
         <v>209</v>
       </c>
       <c r="D3">
-        <v>168</v>
+        <v>5</v>
       </c>
       <c r="E3">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>85</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="M3" s="1">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1110,22 +1110,22 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>180</v>
+        <v>7</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -1148,34 +1148,34 @@
         <v>624</v>
       </c>
       <c r="D5">
-        <v>207</v>
+        <v>10</v>
       </c>
       <c r="E5">
-        <v>414</v>
+        <v>58</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>82</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>96</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L5">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="M5" s="1">
-        <v>100</v>
+        <v>99.7</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1186,25 +1186,25 @@
         <v>15</v>
       </c>
       <c r="C6">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D6">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E6">
-        <v>135</v>
+        <v>45</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>70</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="I6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -1213,7 +1213,7 @@
         <v>0</v>
       </c>
       <c r="L6">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="M6" s="1">
         <v>100</v>
@@ -1230,22 +1230,22 @@
         <v>138</v>
       </c>
       <c r="D7">
-        <v>88</v>
+        <v>14</v>
       </c>
       <c r="E7">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -1274,22 +1274,22 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>112</v>
+        <v>8</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="I8">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -1309,34 +1309,34 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D9">
-        <v>118</v>
+        <v>18</v>
       </c>
       <c r="E9">
-        <v>293</v>
+        <v>88</v>
       </c>
       <c r="F9">
-        <v>3</v>
+        <v>145</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="H9">
-        <v>4</v>
+        <v>79</v>
       </c>
       <c r="I9">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K9">
         <v>0</v>
       </c>
       <c r="L9">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="M9" s="1">
         <v>100</v>
@@ -1347,37 +1347,37 @@
         <v>13</v>
       </c>
       <c r="C10">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="D10">
-        <v>325</v>
+        <v>28</v>
       </c>
       <c r="E10">
-        <v>707</v>
+        <v>146</v>
       </c>
       <c r="F10">
-        <v>3</v>
+        <v>337</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>141</v>
       </c>
       <c r="H10">
-        <v>6</v>
+        <v>175</v>
       </c>
       <c r="I10">
-        <v>5</v>
+        <v>163</v>
       </c>
       <c r="J10">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L10">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="M10" s="1">
-        <v>100</v>
+        <v>99.8</v>
       </c>
     </row>
   </sheetData>
@@ -1451,28 +1451,28 @@
         <v>4</v>
       </c>
       <c r="F2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I2">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J2">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="L2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="M2" s="1">
-        <v>35.3</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1492,28 +1492,28 @@
         <v>7</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3">
         <v>8</v>
       </c>
       <c r="H3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I3">
         <v>14</v>
       </c>
       <c r="J3">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K3">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L3">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M3" s="1">
-        <v>40.7</v>
+        <v>41.1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1536,25 +1536,25 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J4">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="K4">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="L4">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="M4" s="1">
-        <v>35</v>
+        <v>27.2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1574,28 +1574,28 @@
         <v>11</v>
       </c>
       <c r="F5">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G5">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H5">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="I5">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J5">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="K5">
-        <v>393</v>
+        <v>407</v>
       </c>
       <c r="L5">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="M5" s="1">
-        <v>37</v>
+        <v>34.8</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1606,37 +1606,37 @@
         <v>15</v>
       </c>
       <c r="C6">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F6">
+        <v>18</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
         <v>14</v>
       </c>
-      <c r="G6">
-        <v>10</v>
-      </c>
-      <c r="H6">
-        <v>16</v>
-      </c>
       <c r="I6">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="J6">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K6">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="L6">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="M6" s="1">
-        <v>65.5</v>
+        <v>63.4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1650,34 +1650,34 @@
         <v>138</v>
       </c>
       <c r="D7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E7">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F7">
+        <v>7</v>
+      </c>
+      <c r="G7">
         <v>6</v>
       </c>
-      <c r="G7">
-        <v>9</v>
-      </c>
       <c r="H7">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J7">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="K7">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="L7">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M7" s="1">
-        <v>59.4</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1697,28 +1697,28 @@
         <v>4</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H8">
+        <v>14</v>
+      </c>
+      <c r="I8">
         <v>12</v>
-      </c>
-      <c r="I8">
-        <v>15</v>
       </c>
       <c r="J8">
         <v>28</v>
       </c>
       <c r="K8">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L8">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M8" s="1">
-        <v>55.2</v>
+        <v>54.3</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1729,37 +1729,37 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E9">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F9">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G9">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H9">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I9">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="J9">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="K9">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="L9">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="M9" s="1">
-        <v>60.7</v>
+        <v>60.1</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1767,37 +1767,37 @@
         <v>13</v>
       </c>
       <c r="C10">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="D10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E10">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="F10">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="G10">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H10">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="I10">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="J10">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="K10">
-        <v>560</v>
+        <v>577</v>
       </c>
       <c r="L10">
-        <v>489</v>
+        <v>473</v>
       </c>
       <c r="M10" s="1">
-        <v>46.6</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1874,10 +1874,10 @@
         <v>1</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J2">
         <v>23</v>
@@ -1906,25 +1906,25 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3">
         <v>2</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L3" s="1">
-        <v>23.3</v>
+        <v>20.9</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1950,10 +1950,10 @@
         <v>3</v>
       </c>
       <c r="H4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J4">
         <v>20</v>
@@ -2020,25 +2020,25 @@
         <v>1</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G6">
         <v>5</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K6">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L6" s="1">
-        <v>45.9</v>
+        <v>43.2</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -2055,28 +2055,28 @@
         <v>1</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="H7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J7">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K7">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L7" s="1">
-        <v>40.5</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2090,16 +2090,16 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H8">
         <v>3</v>
@@ -2108,13 +2108,13 @@
         <v>4</v>
       </c>
       <c r="J8">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K8">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L8" s="1">
-        <v>45.2</v>
+        <v>48.4</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2131,28 +2131,28 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9">
         <v>2</v>
       </c>
       <c r="I9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J9">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="K9">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L9" s="1">
-        <v>26.2</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -2169,10 +2169,10 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -2207,28 +2207,28 @@
         <v>2</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="K11">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L11" s="1">
-        <v>34.2</v>
+        <v>28.9</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -2242,7 +2242,7 @@
         <v>0</v>
       </c>
       <c r="D12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2254,10 +2254,10 @@
         <v>3</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J12">
         <v>14</v>
@@ -2289,22 +2289,22 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I13">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="J13">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="K13">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="L13" s="1">
-        <v>51.2</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -2327,22 +2327,22 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I14">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J14">
+        <v>16</v>
+      </c>
+      <c r="K14">
         <v>14</v>
       </c>
-      <c r="K14">
-        <v>16</v>
-      </c>
       <c r="L14" s="1">
-        <v>53.3</v>
+        <v>46.7</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -2368,19 +2368,19 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15">
         <v>4</v>
       </c>
       <c r="J15">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K15">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L15" s="1">
-        <v>14.7</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -2400,25 +2400,25 @@
         <v>0</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16">
+        <v>9</v>
+      </c>
+      <c r="J16">
+        <v>8</v>
+      </c>
+      <c r="K16">
         <v>12</v>
       </c>
-      <c r="J16">
-        <v>6</v>
-      </c>
-      <c r="K16">
-        <v>14</v>
-      </c>
       <c r="L16" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -2444,19 +2444,19 @@
         <v>0</v>
       </c>
       <c r="H17">
+        <v>2</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17">
+        <v>33</v>
+      </c>
+      <c r="K17">
         <v>3</v>
       </c>
-      <c r="I17">
-        <v>3</v>
-      </c>
-      <c r="J17">
-        <v>30</v>
-      </c>
-      <c r="K17">
-        <v>6</v>
-      </c>
       <c r="L17" s="1">
-        <v>16.7</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -2485,16 +2485,16 @@
         <v>7</v>
       </c>
       <c r="I18">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J18">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="K18">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="L18" s="1">
-        <v>67.90000000000001</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -2523,16 +2523,16 @@
         <v>0</v>
       </c>
       <c r="I19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J19">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L19" s="1">
-        <v>9.4</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -2546,31 +2546,31 @@
         <v>0</v>
       </c>
       <c r="D20">
+        <v>5</v>
+      </c>
+      <c r="E20">
+        <v>6</v>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+      <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="H20">
         <v>4</v>
       </c>
-      <c r="E20">
-        <v>7</v>
-      </c>
-      <c r="F20">
-        <v>2</v>
-      </c>
-      <c r="G20">
-        <v>2</v>
-      </c>
-      <c r="H20">
-        <v>3</v>
-      </c>
       <c r="I20">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K20">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L20" s="1">
-        <v>84.8</v>
+        <v>81.8</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -2587,7 +2587,7 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F21">
         <v>4</v>
@@ -2596,10 +2596,10 @@
         <v>6</v>
       </c>
       <c r="H21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I21">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J21">
         <v>15</v>
@@ -2622,31 +2622,31 @@
         <v>1</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G22">
+        <v>4</v>
+      </c>
+      <c r="H22">
         <v>5</v>
-      </c>
-      <c r="H22">
-        <v>7</v>
       </c>
       <c r="I22">
         <v>9</v>
       </c>
       <c r="J22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K22">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L22" s="1">
-        <v>90</v>
+        <v>86.7</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -2654,7 +2654,7 @@
         <v>38</v>
       </c>
       <c r="B23">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -2663,7 +2663,7 @@
         <v>1</v>
       </c>
       <c r="E23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -2681,10 +2681,10 @@
         <v>22</v>
       </c>
       <c r="K23">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L23" s="1">
-        <v>33.3</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -2704,25 +2704,25 @@
         <v>0</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H24">
+        <v>4</v>
+      </c>
+      <c r="I24">
         <v>11</v>
       </c>
-      <c r="I24">
-        <v>6</v>
-      </c>
       <c r="J24">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K24">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L24" s="1">
-        <v>57.6</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -2736,13 +2736,13 @@
         <v>0</v>
       </c>
       <c r="D25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E25">
         <v>1</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25">
         <v>2</v>
@@ -2751,16 +2751,16 @@
         <v>3</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J25">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K25">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L25" s="1">
-        <v>57.6</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -2771,10 +2771,10 @@
         <v>36</v>
       </c>
       <c r="C26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26">
         <v>2</v>
@@ -2783,22 +2783,22 @@
         <v>1</v>
       </c>
       <c r="G26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H26">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I26">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J26">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K26">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="L26" s="1">
-        <v>58.3</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -2815,16 +2815,16 @@
         <v>3</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27">
+        <v>3</v>
+      </c>
+      <c r="G27">
         <v>4</v>
       </c>
-      <c r="G27">
-        <v>2</v>
-      </c>
       <c r="H27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I27">
         <v>2</v>
@@ -2850,7 +2850,7 @@
         <v>0</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28">
         <v>2</v>
@@ -2862,7 +2862,7 @@
         <v>3</v>
       </c>
       <c r="H28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I28">
         <v>11</v>
@@ -2894,13 +2894,13 @@
         <v>0</v>
       </c>
       <c r="F29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29">
+        <v>2</v>
+      </c>
+      <c r="H29">
         <v>3</v>
-      </c>
-      <c r="H29">
-        <v>1</v>
       </c>
       <c r="I29">
         <v>1</v>
@@ -2929,19 +2929,19 @@
         <v>3</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F30">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G30">
         <v>3</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I30">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J30">
         <v>7</v>
@@ -2973,22 +2973,22 @@
         <v>0</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I31">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J31">
+        <v>14</v>
+      </c>
+      <c r="K31">
         <v>12</v>
       </c>
-      <c r="K31">
-        <v>14</v>
-      </c>
       <c r="L31" s="1">
-        <v>53.8</v>
+        <v>46.2</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -3011,22 +3011,22 @@
         <v>0</v>
       </c>
       <c r="G32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H32">
         <v>5</v>
       </c>
       <c r="I32">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K32">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L32" s="1">
-        <v>58.8</v>
+        <v>64.7</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -3049,22 +3049,22 @@
         <v>0</v>
       </c>
       <c r="G33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H33">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I33">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J33">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="K33">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="L33" s="1">
-        <v>51.6</v>
+        <v>41.9</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -3084,25 +3084,25 @@
         <v>0</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34">
         <v>3</v>
       </c>
       <c r="H34">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I34">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J34">
+        <v>8</v>
+      </c>
+      <c r="K34">
         <v>11</v>
       </c>
-      <c r="K34">
-        <v>8</v>
-      </c>
       <c r="L34" s="1">
-        <v>42.1</v>
+        <v>57.9</v>
       </c>
     </row>
   </sheetData>
@@ -3184,7 +3184,7 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="1">
         <v>76.7</v>
@@ -3193,7 +3193,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="1">
-        <v>76.7</v>
+        <v>79.09999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -3256,22 +3256,22 @@
         <v>37</v>
       </c>
       <c r="C6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F6" s="1">
-        <v>54.1</v>
+        <v>56.8</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
       </c>
       <c r="H6" s="1">
-        <v>54.1</v>
+        <v>56.8</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -3288,7 +3288,7 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F7" s="1">
         <v>59.5</v>
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="1">
-        <v>59.5</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -3314,7 +3314,7 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F8" s="1">
         <v>54.8</v>
@@ -3323,7 +3323,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="1">
-        <v>54.8</v>
+        <v>51.6</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3337,19 +3337,19 @@
         <v>31</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F9" s="1">
         <v>73.8</v>
       </c>
       <c r="G9" s="1">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="H9" s="1">
-        <v>73.8</v>
+        <v>78.59999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -3392,7 +3392,7 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F11" s="1">
         <v>65.8</v>
@@ -3401,7 +3401,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="1">
-        <v>65.8</v>
+        <v>71.09999999999999</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -3415,7 +3415,7 @@
         <v>14</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12">
         <v>14</v>
@@ -3424,7 +3424,7 @@
         <v>48.3</v>
       </c>
       <c r="G12" s="1">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="H12" s="1">
         <v>48.3</v>
@@ -3444,7 +3444,7 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F13" s="1">
         <v>48.8</v>
@@ -3453,7 +3453,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="1">
-        <v>48.8</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -3470,7 +3470,7 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F14" s="1">
         <v>46.7</v>
@@ -3479,7 +3479,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="1">
-        <v>46.7</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -3496,7 +3496,7 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F15" s="1">
         <v>85.3</v>
@@ -3505,7 +3505,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="1">
-        <v>85.3</v>
+        <v>88.2</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -3522,7 +3522,7 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F16" s="1">
         <v>30</v>
@@ -3531,7 +3531,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="1">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -3548,7 +3548,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F17" s="1">
         <v>83.3</v>
@@ -3557,7 +3557,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="1">
-        <v>83.3</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -3574,7 +3574,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F18" s="1">
         <v>32.1</v>
@@ -3583,7 +3583,7 @@
         <v>0</v>
       </c>
       <c r="H18" s="1">
-        <v>32.1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -3600,7 +3600,7 @@
         <v>0</v>
       </c>
       <c r="E19">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F19" s="1">
         <v>90.59999999999999</v>
@@ -3609,7 +3609,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="1">
-        <v>90.59999999999999</v>
+        <v>93.8</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -3626,7 +3626,7 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F20" s="1">
         <v>15.2</v>
@@ -3635,7 +3635,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="1">
-        <v>15.2</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -3678,7 +3678,7 @@
         <v>0</v>
       </c>
       <c r="E22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F22" s="1">
         <v>10</v>
@@ -3687,7 +3687,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="1">
-        <v>10</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -3695,7 +3695,7 @@
         <v>38</v>
       </c>
       <c r="B23">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C23">
         <v>22</v>
@@ -3707,13 +3707,13 @@
         <v>22</v>
       </c>
       <c r="F23" s="1">
-        <v>66.7</v>
+        <v>64.7</v>
       </c>
       <c r="G23" s="1">
         <v>0</v>
       </c>
       <c r="H23" s="1">
-        <v>66.7</v>
+        <v>64.7</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -3730,7 +3730,7 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F24" s="1">
         <v>42.4</v>
@@ -3739,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="1">
-        <v>42.4</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -3756,7 +3756,7 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F25" s="1">
         <v>42.4</v>
@@ -3765,7 +3765,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="1">
-        <v>42.4</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -3782,7 +3782,7 @@
         <v>0</v>
       </c>
       <c r="E26">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F26" s="1">
         <v>41.7</v>
@@ -3791,7 +3791,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="1">
-        <v>41.7</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -3912,7 +3912,7 @@
         <v>0</v>
       </c>
       <c r="E31">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F31" s="1">
         <v>46.2</v>
@@ -3921,7 +3921,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="1">
-        <v>46.2</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -3938,7 +3938,7 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F32" s="1">
         <v>41.2</v>
@@ -3947,7 +3947,7 @@
         <v>0</v>
       </c>
       <c r="H32" s="1">
-        <v>41.2</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -3964,7 +3964,7 @@
         <v>0</v>
       </c>
       <c r="E33">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F33" s="1">
         <v>48.4</v>
@@ -3973,7 +3973,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="1">
-        <v>48.4</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -3990,7 +3990,7 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F34" s="1">
         <v>57.9</v>
@@ -3999,7 +3999,7 @@
         <v>0</v>
       </c>
       <c r="H34" s="1">
-        <v>57.9</v>
+        <v>42.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Segundo Parcial 16 mayo noche
</commit_message>
<xml_diff>
--- a/Totales Generales.xlsx
+++ b/Totales Generales.xlsx
@@ -775,7 +775,7 @@
         <v>5</v>
       </c>
       <c r="F6">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G6">
         <v>10</v>
@@ -784,7 +784,7 @@
         <v>16</v>
       </c>
       <c r="I6">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J6">
         <v>39</v>
@@ -816,13 +816,13 @@
         <v>8</v>
       </c>
       <c r="F7">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I7">
         <v>13</v>
@@ -898,16 +898,16 @@
         <v>17</v>
       </c>
       <c r="F9">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G9">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H9">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I9">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J9">
         <v>95</v>
@@ -936,16 +936,16 @@
         <v>28</v>
       </c>
       <c r="F10">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G10">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H10">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I10">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J10">
         <v>204</v>
@@ -1025,34 +1025,34 @@
         <v>235</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="F2">
-        <v>161</v>
+        <v>13</v>
       </c>
       <c r="G2">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="L2">
-        <v>235</v>
+        <v>214</v>
       </c>
       <c r="M2" s="1">
-        <v>100</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1069,31 +1069,31 @@
         <v>5</v>
       </c>
       <c r="E3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G3">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="H3">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="I3">
         <v>65</v>
       </c>
       <c r="J3">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>47</v>
       </c>
       <c r="L3">
-        <v>207</v>
+        <v>162</v>
       </c>
       <c r="M3" s="1">
-        <v>99</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1110,31 +1110,31 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F4">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="G4">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="H4">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="I4">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="J4">
+        <v>69</v>
+      </c>
+      <c r="K4">
         <v>30</v>
       </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
       <c r="L4">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="M4" s="1">
-        <v>100</v>
+        <v>83.3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1148,34 +1148,34 @@
         <v>624</v>
       </c>
       <c r="D5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E5">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="F5">
+        <v>31</v>
+      </c>
+      <c r="G5">
+        <v>47</v>
+      </c>
+      <c r="H5">
+        <v>56</v>
+      </c>
+      <c r="I5">
         <v>192</v>
       </c>
-      <c r="G5">
-        <v>82</v>
-      </c>
-      <c r="H5">
-        <v>96</v>
-      </c>
-      <c r="I5">
-        <v>141</v>
-      </c>
       <c r="J5">
-        <v>43</v>
+        <v>172</v>
       </c>
       <c r="K5">
-        <v>2</v>
+        <v>98</v>
       </c>
       <c r="L5">
-        <v>622</v>
+        <v>526</v>
       </c>
       <c r="M5" s="1">
-        <v>99.7</v>
+        <v>84.3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1189,25 +1189,25 @@
         <v>172</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="F6">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="G6">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="H6">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>73</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -1230,25 +1230,25 @@
         <v>138</v>
       </c>
       <c r="D7">
+        <v>11</v>
+      </c>
+      <c r="E7">
         <v>14</v>
       </c>
-      <c r="E7">
-        <v>35</v>
-      </c>
       <c r="F7">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="G7">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="H7">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I7">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -1274,31 +1274,31 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F8">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="G8">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="H8">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I8">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="J8">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="K8">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="L8">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="M8" s="1">
-        <v>100</v>
+        <v>81.90000000000001</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1312,34 +1312,34 @@
         <v>426</v>
       </c>
       <c r="D9">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E9">
-        <v>88</v>
+        <v>41</v>
       </c>
       <c r="F9">
-        <v>145</v>
+        <v>37</v>
       </c>
       <c r="G9">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H9">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I9">
-        <v>22</v>
+        <v>117</v>
       </c>
       <c r="J9">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="K9">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="L9">
-        <v>426</v>
+        <v>405</v>
       </c>
       <c r="M9" s="1">
-        <v>100</v>
+        <v>95.09999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1350,34 +1350,34 @@
         <v>1050</v>
       </c>
       <c r="D10">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E10">
-        <v>146</v>
+        <v>63</v>
       </c>
       <c r="F10">
-        <v>337</v>
+        <v>68</v>
       </c>
       <c r="G10">
-        <v>141</v>
+        <v>103</v>
       </c>
       <c r="H10">
-        <v>175</v>
+        <v>140</v>
       </c>
       <c r="I10">
-        <v>163</v>
+        <v>309</v>
       </c>
       <c r="J10">
-        <v>58</v>
+        <v>229</v>
       </c>
       <c r="K10">
-        <v>2</v>
+        <v>119</v>
       </c>
       <c r="L10">
-        <v>1048</v>
+        <v>931</v>
       </c>
       <c r="M10" s="1">
-        <v>99.8</v>
+        <v>88.7</v>
       </c>
     </row>
   </sheetData>
@@ -1445,34 +1445,34 @@
         <v>235</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F2">
+        <v>8</v>
+      </c>
+      <c r="G2">
         <v>10</v>
       </c>
-      <c r="G2">
-        <v>9</v>
-      </c>
       <c r="H2">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I2">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="J2">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K2">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="M2" s="1">
-        <v>34.9</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1486,25 +1486,25 @@
         <v>209</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G3">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I3">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J3">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K3">
         <v>123</v>
@@ -1542,19 +1542,19 @@
         <v>4</v>
       </c>
       <c r="I4">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J4">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K4">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L4">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M4" s="1">
-        <v>27.2</v>
+        <v>26.7</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1568,22 +1568,22 @@
         <v>624</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E5">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F5">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G5">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="H5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I5">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="J5">
         <v>96</v>
@@ -1615,28 +1615,28 @@
         <v>7</v>
       </c>
       <c r="F6">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G6">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H6">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I6">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J6">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="K6">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="L6">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="M6" s="1">
-        <v>63.4</v>
+        <v>58.7</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1653,31 +1653,31 @@
         <v>4</v>
       </c>
       <c r="E7">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F7">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H7">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I7">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J7">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K7">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="L7">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M7" s="1">
-        <v>60.9</v>
+        <v>60.1</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1697,28 +1697,28 @@
         <v>4</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I8">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J8">
         <v>28</v>
       </c>
       <c r="K8">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L8">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M8" s="1">
-        <v>54.3</v>
+        <v>53.4</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1735,31 +1735,31 @@
         <v>5</v>
       </c>
       <c r="E9">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F9">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G9">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="H9">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="I9">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J9">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="K9">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="L9">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="M9" s="1">
-        <v>60.1</v>
+        <v>57.7</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1770,34 +1770,34 @@
         <v>1050</v>
       </c>
       <c r="D10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E10">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F10">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G10">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="H10">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I10">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J10">
-        <v>195</v>
+        <v>179</v>
       </c>
       <c r="K10">
-        <v>577</v>
+        <v>587</v>
       </c>
       <c r="L10">
-        <v>473</v>
+        <v>463</v>
       </c>
       <c r="M10" s="1">
-        <v>45</v>
+        <v>44.1</v>
       </c>
     </row>
   </sheetData>
@@ -1865,7 +1865,7 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -1874,7 +1874,7 @@
         <v>1</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I2">
         <v>4</v>
@@ -1903,7 +1903,7 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -1915,7 +1915,7 @@
         <v>2</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J3">
         <v>34</v>
@@ -1935,34 +1935,34 @@
         <v>39</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
         <v>3</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
       </c>
       <c r="G4">
         <v>3</v>
       </c>
       <c r="H4">
+        <v>6</v>
+      </c>
+      <c r="I4">
         <v>5</v>
       </c>
-      <c r="I4">
-        <v>7</v>
-      </c>
       <c r="J4">
+        <v>19</v>
+      </c>
+      <c r="K4">
         <v>20</v>
       </c>
-      <c r="K4">
-        <v>19</v>
-      </c>
       <c r="L4" s="1">
-        <v>48.7</v>
+        <v>51.3</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1979,13 +1979,13 @@
         <v>2</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1994,13 +1994,13 @@
         <v>5</v>
       </c>
       <c r="J5">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K5">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L5" s="1">
-        <v>22.5</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -2014,13 +2014,13 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6">
         <v>1</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6">
         <v>5</v>
@@ -2052,31 +2052,31 @@
         <v>0</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J7">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K7">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L7" s="1">
-        <v>42.9</v>
+        <v>38.1</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2143,16 +2143,16 @@
         <v>2</v>
       </c>
       <c r="I9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J9">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L9" s="1">
-        <v>21.4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -2169,10 +2169,10 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -2239,7 +2239,7 @@
         <v>29</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12">
         <v>2</v>
@@ -2248,25 +2248,25 @@
         <v>1</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J12">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K12">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L12" s="1">
-        <v>51.7</v>
+        <v>55.2</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -2280,19 +2280,19 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13">
         <v>0</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I13">
         <v>17</v>
@@ -2444,19 +2444,19 @@
         <v>0</v>
       </c>
       <c r="H17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J17">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L17" s="1">
-        <v>8.300000000000001</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -2549,19 +2549,19 @@
         <v>5</v>
       </c>
       <c r="E20">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G20">
         <v>2</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I20">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J20">
         <v>6</v>
@@ -2587,28 +2587,28 @@
         <v>0</v>
       </c>
       <c r="E21">
+        <v>2</v>
+      </c>
+      <c r="F21">
+        <v>8</v>
+      </c>
+      <c r="G21">
         <v>5</v>
-      </c>
-      <c r="F21">
-        <v>4</v>
-      </c>
-      <c r="G21">
-        <v>6</v>
       </c>
       <c r="H21">
         <v>5</v>
       </c>
       <c r="I21">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J21">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="K21">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="L21" s="1">
-        <v>64.3</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -2622,31 +2622,31 @@
         <v>1</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>7</v>
+      </c>
+      <c r="I22">
         <v>4</v>
       </c>
-      <c r="H22">
-        <v>5</v>
-      </c>
-      <c r="I22">
+      <c r="J22">
         <v>9</v>
       </c>
-      <c r="J22">
-        <v>4</v>
-      </c>
       <c r="K22">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="L22" s="1">
-        <v>86.7</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -2660,31 +2660,31 @@
         <v>0</v>
       </c>
       <c r="D23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23">
         <v>2</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23">
         <v>1</v>
       </c>
       <c r="H23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I23">
         <v>5</v>
       </c>
       <c r="J23">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K23">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L23" s="1">
-        <v>35.3</v>
+        <v>38.2</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -2707,13 +2707,13 @@
         <v>1</v>
       </c>
       <c r="G24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I24">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J24">
         <v>16</v>
@@ -2736,10 +2736,10 @@
         <v>0</v>
       </c>
       <c r="D25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -2751,16 +2751,16 @@
         <v>3</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J25">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K25">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L25" s="1">
-        <v>54.5</v>
+        <v>57.6</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -2774,22 +2774,22 @@
         <v>2</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E26">
         <v>2</v>
       </c>
       <c r="F26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J26">
         <v>12</v>
@@ -2821,10 +2821,10 @@
         <v>3</v>
       </c>
       <c r="G27">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I27">
         <v>2</v>
@@ -2850,31 +2850,31 @@
         <v>0</v>
       </c>
       <c r="D28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28">
         <v>0</v>
       </c>
       <c r="I28">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J28">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K28">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L28" s="1">
-        <v>60</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -2900,19 +2900,19 @@
         <v>2</v>
       </c>
       <c r="H29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I29">
         <v>1</v>
       </c>
       <c r="J29">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K29">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L29" s="1">
-        <v>42.9</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -2935,10 +2935,10 @@
         <v>2</v>
       </c>
       <c r="G30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I30">
         <v>3</v>
@@ -2979,16 +2979,16 @@
         <v>2</v>
       </c>
       <c r="I31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J31">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K31">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L31" s="1">
-        <v>46.2</v>
+        <v>42.3</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -3014,10 +3014,10 @@
         <v>1</v>
       </c>
       <c r="H32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J32">
         <v>6</v>
@@ -3081,16 +3081,16 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34">
         <v>3</v>
       </c>
       <c r="H34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I34">
         <v>6</v>
@@ -3210,7 +3210,7 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F4" s="1">
         <v>51.3</v>
@@ -3219,7 +3219,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="1">
-        <v>51.3</v>
+        <v>48.7</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -3236,7 +3236,7 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F5" s="1">
         <v>77.5</v>
@@ -3245,7 +3245,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="1">
-        <v>77.5</v>
+        <v>72.5</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3259,7 +3259,7 @@
         <v>21</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E6">
         <v>21</v>
@@ -3268,7 +3268,7 @@
         <v>56.8</v>
       </c>
       <c r="G6" s="1">
-        <v>0</v>
+        <v>56.8</v>
       </c>
       <c r="H6" s="1">
         <v>56.8</v>
@@ -3288,7 +3288,7 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F7" s="1">
         <v>59.5</v>
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="1">
-        <v>57.1</v>
+        <v>61.9</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -3337,19 +3337,19 @@
         <v>31</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="E9">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F9" s="1">
         <v>73.8</v>
       </c>
       <c r="G9" s="1">
-        <v>2.4</v>
+        <v>81</v>
       </c>
       <c r="H9" s="1">
-        <v>78.59999999999999</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -3415,19 +3415,19 @@
         <v>14</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E12">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F12" s="1">
         <v>48.3</v>
       </c>
       <c r="G12" s="1">
-        <v>3.4</v>
+        <v>44.8</v>
       </c>
       <c r="H12" s="1">
-        <v>48.3</v>
+        <v>44.8</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -3548,7 +3548,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F17" s="1">
         <v>83.3</v>
@@ -3557,7 +3557,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="1">
-        <v>91.7</v>
+        <v>94.40000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -3597,7 +3597,7 @@
         <v>29</v>
       </c>
       <c r="D19">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E19">
         <v>30</v>
@@ -3606,7 +3606,7 @@
         <v>90.59999999999999</v>
       </c>
       <c r="G19" s="1">
-        <v>0</v>
+        <v>93.8</v>
       </c>
       <c r="H19" s="1">
         <v>93.8</v>
@@ -3652,7 +3652,7 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F21" s="1">
         <v>35.7</v>
@@ -3661,7 +3661,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="1">
-        <v>35.7</v>
+        <v>45.2</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -3678,7 +3678,7 @@
         <v>0</v>
       </c>
       <c r="E22">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F22" s="1">
         <v>10</v>
@@ -3687,7 +3687,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="1">
-        <v>13.3</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -3704,7 +3704,7 @@
         <v>0</v>
       </c>
       <c r="E23">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F23" s="1">
         <v>64.7</v>
@@ -3713,7 +3713,7 @@
         <v>0</v>
       </c>
       <c r="H23" s="1">
-        <v>64.7</v>
+        <v>61.8</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -3756,7 +3756,7 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F25" s="1">
         <v>42.4</v>
@@ -3765,7 +3765,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="1">
-        <v>45.5</v>
+        <v>42.4</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -3834,7 +3834,7 @@
         <v>0</v>
       </c>
       <c r="E28">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F28" s="1">
         <v>40</v>
@@ -3843,7 +3843,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="1">
-        <v>40</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -3860,7 +3860,7 @@
         <v>0</v>
       </c>
       <c r="E29">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F29" s="1">
         <v>57.1</v>
@@ -3869,7 +3869,7 @@
         <v>0</v>
       </c>
       <c r="H29" s="1">
-        <v>57.1</v>
+        <v>64.3</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -3883,7 +3883,7 @@
         <v>7</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E30">
         <v>7</v>
@@ -3892,7 +3892,7 @@
         <v>30.4</v>
       </c>
       <c r="G30" s="1">
-        <v>0</v>
+        <v>30.4</v>
       </c>
       <c r="H30" s="1">
         <v>30.4</v>
@@ -3912,7 +3912,7 @@
         <v>0</v>
       </c>
       <c r="E31">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F31" s="1">
         <v>46.2</v>
@@ -3921,7 +3921,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="1">
-        <v>53.8</v>
+        <v>57.7</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -3935,7 +3935,7 @@
         <v>7</v>
       </c>
       <c r="D32">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E32">
         <v>6</v>
@@ -3944,7 +3944,7 @@
         <v>41.2</v>
       </c>
       <c r="G32" s="1">
-        <v>0</v>
+        <v>35.3</v>
       </c>
       <c r="H32" s="1">
         <v>35.3</v>
@@ -3987,7 +3987,7 @@
         <v>11</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E34">
         <v>8</v>
@@ -3996,7 +3996,7 @@
         <v>57.9</v>
       </c>
       <c r="G34" s="1">
-        <v>0</v>
+        <v>42.1</v>
       </c>
       <c r="H34" s="1">
         <v>42.1</v>

</xml_diff>